<commit_message>
Preenche tamanho dos rótulos B2C em PET âmbar com vinil/BOPP
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018k4AWMEfPQ3PeJhEoKFmKz
</commit_message>
<xml_diff>
--- a/Rotulos_Consolidado_atualizado.xlsx
+++ b/Rotulos_Consolidado_atualizado.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="931" uniqueCount="82">
   <si>
     <t xml:space="preserve">Necessidade de rótulos – consolidado</t>
   </si>
@@ -92,6 +92,9 @@
     <t xml:space="preserve">Vinil ou Bopp</t>
   </si>
   <si>
+    <t xml:space="preserve">18 x 6,5 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">Vidro square cristal / válvula spray prata 28/410</t>
   </si>
   <si>
@@ -104,33 +107,30 @@
     <t xml:space="preserve">Aromatizador (Refil)</t>
   </si>
   <si>
+    <t xml:space="preserve">22 x 8 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fragrância Concentrada</t>
   </si>
   <si>
     <t xml:space="preserve">Fragrância Concentrada (Refil Equipamento)</t>
   </si>
   <si>
+    <t xml:space="preserve">13 x 5 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bamboo</t>
   </si>
   <si>
-    <t xml:space="preserve">Não informado</t>
-  </si>
-  <si>
     <t xml:space="preserve">B2B</t>
   </si>
   <si>
-    <t xml:space="preserve">22 x 8 cm</t>
-  </si>
-  <si>
     <t xml:space="preserve">28 x 10,5 cm</t>
   </si>
   <si>
     <t xml:space="preserve">Fragrância Ultra Concentrada</t>
   </si>
   <si>
-    <t xml:space="preserve">13 x 5 cm</t>
-  </si>
-  <si>
     <t xml:space="preserve">Capim Limão</t>
   </si>
   <si>
@@ -140,9 +140,6 @@
     <t xml:space="preserve">Citric Bath</t>
   </si>
   <si>
-    <t xml:space="preserve">18 x 6,5 cm</t>
-  </si>
-  <si>
     <t xml:space="preserve">Citrus Flowers</t>
   </si>
   <si>
@@ -228,9 +225,6 @@
   </si>
   <si>
     <t xml:space="preserve">Siciliano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silver</t>
   </si>
   <si>
     <t xml:space="preserve">Tobacco</t>
@@ -379,14 +373,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -472,12 +466,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -490,10 +488,6 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -642,12 +636,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Rotulos" displayName="Rotulos" ref="A4:I147" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A4:I147">
-    <filterColumn colId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Rotulos" displayName="Rotulos" ref="A4:I144" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A4:I144">
+    <filterColumn colId="5">
       <filters>
-        <filter val="Vidro square cristal / tampa difusora prata 28/410 + batoque + varetas"/>
-        <filter val="Vidro square cristal / válvula spray prata 28/410"/>
+        <filter val="B2C"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="7">
+      <filters>
+        <filter val="Vinil ou Bopp"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -845,7 +843,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I151"/>
+  <dimension ref="A1:I148"/>
   <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -923,7 +921,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
         <v>11</v>
       </c>
@@ -949,7 +947,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
         <v>11</v>
       </c>
@@ -974,8 +972,11 @@
       <c r="H7" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I7" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
         <v>11</v>
       </c>
@@ -986,10 +987,10 @@
         <v>250</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>15</v>
@@ -1003,7 +1004,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>12</v>
@@ -1027,9 +1028,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>12</v>
@@ -1041,7 +1042,7 @@
         <v>20</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>15</v>
@@ -1052,13 +1053,16 @@
       <c r="H10" s="7" t="s">
         <v>22</v>
       </c>
+      <c r="I10" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>15</v>
@@ -1067,7 +1071,7 @@
         <v>13</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>15</v>
@@ -1079,12 +1083,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>100</v>
@@ -1093,7 +1097,7 @@
         <v>20</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>15</v>
@@ -1104,10 +1108,13 @@
       <c r="H12" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I12" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>17</v>
@@ -1131,9 +1138,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>17</v>
@@ -1156,10 +1163,13 @@
       <c r="H14" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I14" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>17</v>
@@ -1168,10 +1178,10 @@
         <v>250</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>15</v>
@@ -1185,10 +1195,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="C16" s="4" t="n">
         <v>400</v>
@@ -1196,11 +1206,11 @@
       <c r="D16" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="8" t="s">
-        <v>30</v>
+      <c r="E16" s="4" t="s">
+        <v>29</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G16" s="6" t="n">
         <v>1</v>
@@ -1209,15 +1219,15 @@
         <v>22</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="C17" s="4" t="n">
         <v>1000</v>
@@ -1225,11 +1235,11 @@
       <c r="D17" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E17" s="8" t="s">
-        <v>30</v>
+      <c r="E17" s="4" t="s">
+        <v>29</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G17" s="6" t="n">
         <v>1</v>
@@ -1238,15 +1248,15 @@
         <v>22</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C18" s="4" t="n">
         <v>100</v>
@@ -1254,11 +1264,11 @@
       <c r="D18" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="8" t="s">
-        <v>30</v>
+      <c r="E18" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G18" s="6" t="n">
         <v>4</v>
@@ -1267,15 +1277,15 @@
         <v>22</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C19" s="4" t="n">
         <v>500</v>
@@ -1283,11 +1293,11 @@
       <c r="D19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E19" s="8" t="s">
-        <v>30</v>
+      <c r="E19" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G19" s="6" t="n">
         <v>2</v>
@@ -1296,12 +1306,12 @@
         <v>22</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>12</v>
@@ -1325,9 +1335,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>12</v>
@@ -1339,7 +1349,7 @@
         <v>20</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>15</v>
@@ -1350,13 +1360,16 @@
       <c r="H21" s="7" t="s">
         <v>22</v>
       </c>
+      <c r="I21" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="C22" s="4" t="n">
         <v>15</v>
@@ -1365,7 +1378,7 @@
         <v>13</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>15</v>
@@ -1377,12 +1390,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="C23" s="4" t="n">
         <v>100</v>
@@ -1391,7 +1404,7 @@
         <v>20</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F23" s="5" t="s">
         <v>15</v>
@@ -1402,10 +1415,13 @@
       <c r="H23" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I23" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>17</v>
@@ -1429,9 +1445,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>17</v>
@@ -1454,10 +1470,13 @@
       <c r="H25" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I25" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>17</v>
@@ -1466,10 +1485,10 @@
         <v>250</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>15</v>
@@ -1486,7 +1505,7 @@
         <v>36</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C27" s="4" t="n">
         <v>100</v>
@@ -1494,11 +1513,12 @@
       <c r="D27" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E27" s="8" t="s">
-        <v>30</v>
+      <c r="E27" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G27" s="6" t="n">
         <v>5</v>
@@ -1507,7 +1527,7 @@
         <v>22</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1536,7 +1556,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
         <v>36</v>
       </c>
@@ -1550,7 +1570,7 @@
         <v>20</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F29" s="5" t="s">
         <v>15</v>
@@ -1560,6 +1580,9 @@
       </c>
       <c r="H29" s="7" t="s">
         <v>22</v>
+      </c>
+      <c r="I29" s="8" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1567,7 +1590,7 @@
         <v>36</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C30" s="4" t="n">
         <v>15</v>
@@ -1576,7 +1599,7 @@
         <v>13</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F30" s="5" t="s">
         <v>15</v>
@@ -1588,12 +1611,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
         <v>36</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C31" s="4" t="n">
         <v>100</v>
@@ -1602,7 +1625,7 @@
         <v>20</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>15</v>
@@ -1613,8 +1636,11 @@
       <c r="H31" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I31" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
         <v>36</v>
       </c>
@@ -1640,7 +1666,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
         <v>36</v>
       </c>
@@ -1665,8 +1691,11 @@
       <c r="H33" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I33" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
         <v>36</v>
       </c>
@@ -1677,10 +1706,10 @@
         <v>250</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F34" s="5" t="s">
         <v>15</v>
@@ -1697,7 +1726,7 @@
         <v>37</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C35" s="4" t="n">
         <v>100</v>
@@ -1705,11 +1734,12 @@
       <c r="D35" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E35" s="8" t="s">
-        <v>30</v>
+      <c r="E35" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G35" s="6" t="n">
         <v>2</v>
@@ -1718,7 +1748,7 @@
         <v>22</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1747,7 +1777,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
         <v>37</v>
       </c>
@@ -1761,7 +1791,7 @@
         <v>20</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F37" s="5" t="s">
         <v>15</v>
@@ -1771,6 +1801,9 @@
       </c>
       <c r="H37" s="7" t="s">
         <v>22</v>
+      </c>
+      <c r="I37" s="8" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1778,7 +1811,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C38" s="4" t="n">
         <v>15</v>
@@ -1787,7 +1820,7 @@
         <v>13</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F38" s="5" t="s">
         <v>15</v>
@@ -1799,12 +1832,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
         <v>37</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C39" s="4" t="n">
         <v>100</v>
@@ -1813,7 +1846,7 @@
         <v>20</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F39" s="5" t="s">
         <v>15</v>
@@ -1824,8 +1857,11 @@
       <c r="H39" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I39" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
         <v>37</v>
       </c>
@@ -1851,7 +1887,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
         <v>37</v>
       </c>
@@ -1876,8 +1912,11 @@
       <c r="H41" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I41" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
         <v>37</v>
       </c>
@@ -1888,10 +1927,10 @@
         <v>250</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F42" s="5" t="s">
         <v>15</v>
@@ -1916,11 +1955,12 @@
       <c r="D43" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E43" s="8" t="s">
-        <v>30</v>
+      <c r="E43" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Aromatizador de Ambientes</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G43" s="6" t="n">
         <v>3</v>
@@ -1929,7 +1969,7 @@
         <v>22</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1937,7 +1977,7 @@
         <v>38</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C44" s="4" t="n">
         <v>1000</v>
@@ -1945,11 +1985,12 @@
       <c r="D44" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E44" s="8" t="s">
-        <v>30</v>
+      <c r="E44" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G44" s="6" t="n">
         <v>4</v>
@@ -1958,15 +1999,15 @@
         <v>22</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C45" s="4" t="n">
         <v>400</v>
@@ -1974,11 +2015,12 @@
       <c r="D45" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E45" s="8" t="s">
-        <v>30</v>
+      <c r="E45" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G45" s="6" t="n">
         <v>2</v>
@@ -1987,15 +2029,15 @@
         <v>22</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C46" s="4" t="n">
         <v>1000</v>
@@ -2003,11 +2045,12 @@
       <c r="D46" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E46" s="8" t="s">
-        <v>30</v>
+      <c r="E46" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G46" s="6" t="n">
         <v>1</v>
@@ -2016,12 +2059,12 @@
         <v>22</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>12</v>
@@ -2045,9 +2088,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>17</v>
@@ -2071,9 +2114,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>17</v>
@@ -2096,10 +2139,13 @@
       <c r="H49" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I49" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>17</v>
@@ -2108,10 +2154,10 @@
         <v>250</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F50" s="5" t="s">
         <v>15</v>
@@ -2125,10 +2171,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C51" s="4" t="n">
         <v>400</v>
@@ -2136,11 +2182,12 @@
       <c r="D51" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E51" s="8" t="s">
-        <v>30</v>
+      <c r="E51" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G51" s="6" t="n">
         <v>3</v>
@@ -2149,15 +2196,15 @@
         <v>22</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C52" s="4" t="n">
         <v>100</v>
@@ -2165,11 +2212,12 @@
       <c r="D52" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E52" s="8" t="s">
-        <v>30</v>
+      <c r="E52" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G52" s="6" t="n">
         <v>1</v>
@@ -2178,15 +2226,15 @@
         <v>22</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C53" s="4" t="n">
         <v>500</v>
@@ -2194,11 +2242,12 @@
       <c r="D53" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E53" s="8" t="s">
-        <v>30</v>
+      <c r="E53" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G53" s="6" t="n">
         <v>13</v>
@@ -2207,15 +2256,15 @@
         <v>22</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C54" s="4" t="n">
         <v>1000</v>
@@ -2223,11 +2272,12 @@
       <c r="D54" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E54" s="8" t="s">
-        <v>30</v>
+      <c r="E54" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G54" s="6" t="n">
         <v>1</v>
@@ -2236,12 +2286,12 @@
         <v>22</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>17</v>
@@ -2252,9 +2302,9 @@
       <c r="D55" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E55" s="8"/>
+      <c r="E55" s="10"/>
       <c r="F55" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G55" s="6" t="n">
         <v>8</v>
@@ -2263,12 +2313,12 @@
         <v>22</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>12</v>
@@ -2292,9 +2342,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>12</v>
@@ -2306,7 +2356,7 @@
         <v>20</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F57" s="5" t="s">
         <v>15</v>
@@ -2317,13 +2367,16 @@
       <c r="H57" s="7" t="s">
         <v>22</v>
       </c>
+      <c r="I57" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C58" s="4" t="n">
         <v>15</v>
@@ -2332,7 +2385,7 @@
         <v>13</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F58" s="5" t="s">
         <v>15</v>
@@ -2344,12 +2397,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C59" s="4" t="n">
         <v>100</v>
@@ -2358,7 +2411,7 @@
         <v>20</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F59" s="5" t="s">
         <v>15</v>
@@ -2369,10 +2422,13 @@
       <c r="H59" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I59" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>17</v>
@@ -2396,9 +2452,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>17</v>
@@ -2421,10 +2477,13 @@
       <c r="H61" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I61" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>17</v>
@@ -2433,10 +2492,10 @@
         <v>250</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F62" s="5" t="s">
         <v>15</v>
@@ -2450,10 +2509,10 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>500</v>
@@ -2461,11 +2520,12 @@
       <c r="D63" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E63" s="8" t="s">
-        <v>30</v>
+      <c r="E63" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F63" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G63" s="6" t="n">
         <v>2</v>
@@ -2474,12 +2534,12 @@
         <v>22</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>12</v>
@@ -2503,9 +2563,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>17</v>
@@ -2529,9 +2589,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>17</v>
@@ -2554,10 +2614,13 @@
       <c r="H66" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I66" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>17</v>
@@ -2566,10 +2629,10 @@
         <v>250</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F67" s="5" t="s">
         <v>15</v>
@@ -2583,10 +2646,10 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B68" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="B68" s="4" t="s">
-        <v>46</v>
       </c>
       <c r="C68" s="4" t="n">
         <v>500</v>
@@ -2594,11 +2657,12 @@
       <c r="D68" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E68" s="8" t="s">
-        <v>30</v>
+      <c r="E68" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Não informada</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G68" s="6" t="n">
         <v>4</v>
@@ -2607,12 +2671,12 @@
         <v>22</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>12</v>
@@ -2623,11 +2687,12 @@
       <c r="D69" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E69" s="8" t="s">
-        <v>30</v>
+      <c r="E69" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Aromatizador de Ambientes</v>
       </c>
       <c r="F69" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G69" s="6" t="n">
         <v>3</v>
@@ -2636,15 +2701,15 @@
         <v>22</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C70" s="4" t="n">
         <v>400</v>
@@ -2652,11 +2717,12 @@
       <c r="D70" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E70" s="8" t="s">
-        <v>30</v>
+      <c r="E70" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G70" s="6" t="n">
         <v>2</v>
@@ -2665,15 +2731,15 @@
         <v>22</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C71" s="4" t="n">
         <v>100</v>
@@ -2681,11 +2747,12 @@
       <c r="D71" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E71" s="8" t="s">
-        <v>30</v>
+      <c r="E71" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F71" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G71" s="6" t="n">
         <v>1</v>
@@ -2694,15 +2761,15 @@
         <v>22</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C72" s="4" t="n">
         <v>500</v>
@@ -2710,11 +2777,12 @@
       <c r="D72" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E72" s="8" t="s">
-        <v>30</v>
+      <c r="E72" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F72" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G72" s="6" t="n">
         <v>3</v>
@@ -2723,15 +2791,15 @@
         <v>22</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C73" s="4" t="n">
         <v>400</v>
@@ -2739,11 +2807,12 @@
       <c r="D73" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E73" s="8" t="s">
-        <v>30</v>
+      <c r="E73" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F73" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G73" s="6" t="n">
         <v>5</v>
@@ -2752,15 +2821,15 @@
         <v>22</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C74" s="4" t="n">
         <v>100</v>
@@ -2768,11 +2837,12 @@
       <c r="D74" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E74" s="8" t="s">
-        <v>30</v>
+      <c r="E74" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F74" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G74" s="6" t="n">
         <v>10</v>
@@ -2781,15 +2851,15 @@
         <v>22</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C75" s="4" t="n">
         <v>1000</v>
@@ -2797,11 +2867,12 @@
       <c r="D75" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E75" s="8" t="s">
-        <v>30</v>
+      <c r="E75" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F75" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G75" s="6" t="n">
         <v>4</v>
@@ -2810,15 +2881,15 @@
         <v>22</v>
       </c>
       <c r="I75" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C76" s="4" t="n">
         <v>400</v>
@@ -2826,11 +2897,12 @@
       <c r="D76" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E76" s="8" t="s">
-        <v>30</v>
+      <c r="E76" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F76" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G76" s="6" t="n">
         <v>8</v>
@@ -2839,15 +2911,15 @@
         <v>22</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>1000</v>
@@ -2855,11 +2927,12 @@
       <c r="D77" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E77" s="8" t="s">
-        <v>30</v>
+      <c r="E77" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F77" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G77" s="6" t="n">
         <v>2</v>
@@ -2868,15 +2941,15 @@
         <v>22</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C78" s="4" t="n">
         <v>100</v>
@@ -2884,11 +2957,12 @@
       <c r="D78" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E78" s="8" t="s">
-        <v>30</v>
+      <c r="E78" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F78" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G78" s="6" t="n">
         <v>28</v>
@@ -2897,15 +2971,15 @@
         <v>22</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>1000</v>
@@ -2913,11 +2987,12 @@
       <c r="D79" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E79" s="8" t="s">
-        <v>30</v>
+      <c r="E79" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F79" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G79" s="6" t="n">
         <v>2</v>
@@ -2926,15 +3001,15 @@
         <v>22</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C80" s="4" t="n">
         <v>100</v>
@@ -2942,11 +3017,12 @@
       <c r="D80" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E80" s="8" t="s">
-        <v>30</v>
+      <c r="E80" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F80" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G80" s="6" t="n">
         <v>34</v>
@@ -2955,15 +3031,15 @@
         <v>22</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>1000</v>
@@ -2971,11 +3047,12 @@
       <c r="D81" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E81" s="8" t="s">
-        <v>30</v>
+      <c r="E81" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F81" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G81" s="6" t="n">
         <v>1</v>
@@ -2984,15 +3061,15 @@
         <v>22</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C82" s="4" t="n">
         <v>400</v>
@@ -3000,11 +3077,12 @@
       <c r="D82" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E82" s="8" t="s">
-        <v>30</v>
+      <c r="E82" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F82" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G82" s="6" t="n">
         <v>6</v>
@@ -3013,15 +3091,15 @@
         <v>22</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C83" s="4" t="n">
         <v>100</v>
@@ -3029,11 +3107,12 @@
       <c r="D83" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E83" s="8" t="s">
-        <v>30</v>
+      <c r="E83" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F83" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G83" s="6" t="n">
         <v>1</v>
@@ -3042,15 +3121,15 @@
         <v>22</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C84" s="4" t="n">
         <v>500</v>
@@ -3058,11 +3137,12 @@
       <c r="D84" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E84" s="8" t="s">
-        <v>30</v>
+      <c r="E84" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F84" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G84" s="6" t="n">
         <v>3</v>
@@ -3071,15 +3151,15 @@
         <v>22</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C85" s="4" t="n">
         <v>1000</v>
@@ -3087,11 +3167,12 @@
       <c r="D85" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E85" s="8" t="s">
-        <v>30</v>
+      <c r="E85" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F85" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G85" s="6" t="n">
         <v>2</v>
@@ -3100,15 +3181,15 @@
         <v>22</v>
       </c>
       <c r="I85" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C86" s="4" t="n">
         <v>1000</v>
@@ -3116,11 +3197,12 @@
       <c r="D86" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E86" s="8" t="s">
-        <v>30</v>
+      <c r="E86" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F86" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G86" s="6" t="n">
         <v>1</v>
@@ -3129,15 +3211,15 @@
         <v>22</v>
       </c>
       <c r="I86" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C87" s="4" t="n">
         <v>400</v>
@@ -3145,11 +3227,12 @@
       <c r="D87" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E87" s="8" t="s">
-        <v>30</v>
+      <c r="E87" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F87" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G87" s="6" t="n">
         <v>6</v>
@@ -3158,15 +3241,15 @@
         <v>22</v>
       </c>
       <c r="I87" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C88" s="4" t="n">
         <v>1000</v>
@@ -3174,11 +3257,12 @@
       <c r="D88" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E88" s="8" t="s">
-        <v>30</v>
+      <c r="E88" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F88" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G88" s="6" t="n">
         <v>5</v>
@@ -3187,15 +3271,15 @@
         <v>22</v>
       </c>
       <c r="I88" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C89" s="4" t="n">
         <v>500</v>
@@ -3203,11 +3287,12 @@
       <c r="D89" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E89" s="8" t="s">
-        <v>30</v>
+      <c r="E89" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F89" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G89" s="6" t="n">
         <v>1</v>
@@ -3216,12 +3301,12 @@
         <v>22</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>12</v>
@@ -3245,9 +3330,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>12</v>
@@ -3259,7 +3344,7 @@
         <v>20</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F91" s="5" t="s">
         <v>15</v>
@@ -3270,13 +3355,16 @@
       <c r="H91" s="7" t="s">
         <v>22</v>
       </c>
+      <c r="I91" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C92" s="4" t="n">
         <v>15</v>
@@ -3285,7 +3373,7 @@
         <v>13</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F92" s="5" t="s">
         <v>15</v>
@@ -3297,12 +3385,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C93" s="4" t="n">
         <v>100</v>
@@ -3311,7 +3399,7 @@
         <v>20</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F93" s="5" t="s">
         <v>15</v>
@@ -3322,10 +3410,13 @@
       <c r="H93" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I93" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>17</v>
@@ -3349,9 +3440,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B95" s="4" t="s">
         <v>17</v>
@@ -3374,10 +3465,13 @@
       <c r="H95" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I95" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>17</v>
@@ -3386,10 +3480,10 @@
         <v>250</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E96" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F96" s="5" t="s">
         <v>15</v>
@@ -3403,7 +3497,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B97" s="4" t="s">
         <v>12</v>
@@ -3427,9 +3521,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B98" s="4" t="s">
         <v>17</v>
@@ -3453,9 +3547,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B99" s="4" t="s">
         <v>17</v>
@@ -3478,10 +3572,13 @@
       <c r="H99" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I99" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B100" s="4" t="s">
         <v>17</v>
@@ -3490,10 +3587,10 @@
         <v>250</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E100" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F100" s="5" t="s">
         <v>15</v>
@@ -3507,10 +3604,10 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C101" s="4" t="n">
         <v>400</v>
@@ -3518,11 +3615,12 @@
       <c r="D101" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E101" s="8" t="s">
-        <v>30</v>
+      <c r="E101" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F101" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G101" s="6" t="n">
         <v>1</v>
@@ -3531,15 +3629,15 @@
         <v>22</v>
       </c>
       <c r="I101" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C102" s="4" t="n">
         <v>100</v>
@@ -3547,11 +3645,12 @@
       <c r="D102" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E102" s="8" t="s">
-        <v>30</v>
+      <c r="E102" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F102" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G102" s="6" t="n">
         <v>1</v>
@@ -3560,15 +3659,15 @@
         <v>22</v>
       </c>
       <c r="I102" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C103" s="4" t="n">
         <v>500</v>
@@ -3576,11 +3675,12 @@
       <c r="D103" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E103" s="8" t="s">
-        <v>30</v>
+      <c r="E103" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F103" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G103" s="6" t="n">
         <v>2</v>
@@ -3589,15 +3689,15 @@
         <v>22</v>
       </c>
       <c r="I103" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C104" s="4" t="n">
         <v>1000</v>
@@ -3605,11 +3705,12 @@
       <c r="D104" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E104" s="8" t="s">
-        <v>30</v>
+      <c r="E104" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F104" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G104" s="6" t="n">
         <v>1</v>
@@ -3618,12 +3719,12 @@
         <v>22</v>
       </c>
       <c r="I104" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B105" s="4" t="s">
         <v>17</v>
@@ -3634,9 +3735,12 @@
       <c r="D105" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E105" s="8"/>
+      <c r="E105" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Perfume para Ambientes</v>
+      </c>
       <c r="F105" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G105" s="6" t="n">
         <v>2</v>
@@ -3645,12 +3749,12 @@
         <v>22</v>
       </c>
       <c r="I105" s="4" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B106" s="4" t="s">
         <v>12</v>
@@ -3661,11 +3765,12 @@
       <c r="D106" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E106" s="8" t="s">
-        <v>30</v>
+      <c r="E106" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Aromatizador de Ambientes</v>
       </c>
       <c r="F106" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G106" s="6" t="n">
         <v>1</v>
@@ -3674,12 +3779,12 @@
         <v>22</v>
       </c>
       <c r="I106" s="4" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B107" s="4" t="s">
         <v>12</v>
@@ -3690,9 +3795,12 @@
       <c r="D107" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E107" s="8"/>
+      <c r="E107" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Aromatizador de Ambientes</v>
+      </c>
       <c r="F107" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G107" s="6" t="n">
         <v>7</v>
@@ -3701,15 +3809,15 @@
         <v>22</v>
       </c>
       <c r="I107" s="4" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C108" s="4" t="n">
         <v>400</v>
@@ -3717,11 +3825,12 @@
       <c r="D108" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E108" s="8" t="s">
-        <v>30</v>
+      <c r="E108" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F108" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G108" s="6" t="n">
         <v>2</v>
@@ -3730,15 +3839,15 @@
         <v>22</v>
       </c>
       <c r="I108" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C109" s="4" t="n">
         <v>100</v>
@@ -3746,11 +3855,12 @@
       <c r="D109" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E109" s="8" t="s">
-        <v>30</v>
+      <c r="E109" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F109" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G109" s="6" t="n">
         <v>1</v>
@@ -3759,12 +3869,12 @@
         <v>22</v>
       </c>
       <c r="I109" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B110" s="4" t="s">
         <v>12</v>
@@ -3788,9 +3898,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B111" s="4" t="s">
         <v>12</v>
@@ -3802,7 +3912,7 @@
         <v>20</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F111" s="5" t="s">
         <v>15</v>
@@ -3813,13 +3923,16 @@
       <c r="H111" s="7" t="s">
         <v>22</v>
       </c>
+      <c r="I111" s="8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C112" s="4" t="n">
         <v>15</v>
@@ -3828,7 +3941,7 @@
         <v>13</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F112" s="5" t="s">
         <v>15</v>
@@ -3840,12 +3953,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C113" s="4" t="n">
         <v>100</v>
@@ -3854,7 +3967,7 @@
         <v>20</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F113" s="5" t="s">
         <v>15</v>
@@ -3865,10 +3978,13 @@
       <c r="H113" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I113" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B114" s="4" t="s">
         <v>17</v>
@@ -3892,9 +4008,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B115" s="4" t="s">
         <v>17</v>
@@ -3917,10 +4033,13 @@
       <c r="H115" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I115" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B116" s="4" t="s">
         <v>17</v>
@@ -3929,10 +4048,10 @@
         <v>250</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F116" s="5" t="s">
         <v>15</v>
@@ -3944,9 +4063,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B117" s="4" t="s">
         <v>17</v>
@@ -3958,7 +4077,7 @@
         <v>20</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F117" s="5" t="s">
         <v>15</v>
@@ -3969,13 +4088,16 @@
       <c r="H117" s="7" t="s">
         <v>22</v>
       </c>
+      <c r="I117" s="8" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C118" s="4" t="n">
         <v>1000</v>
@@ -3983,11 +4105,12 @@
       <c r="D118" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E118" s="8" t="s">
-        <v>30</v>
+      <c r="E118" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F118" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G118" s="6" t="n">
         <v>1</v>
@@ -3996,12 +4119,12 @@
         <v>22</v>
       </c>
       <c r="I118" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B119" s="4" t="s">
         <v>12</v>
@@ -4025,9 +4148,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B120" s="4" t="s">
         <v>17</v>
@@ -4051,9 +4174,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="121" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B121" s="4" t="s">
         <v>17</v>
@@ -4076,10 +4199,13 @@
       <c r="H121" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I121" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B122" s="4" t="s">
         <v>17</v>
@@ -4088,10 +4214,10 @@
         <v>250</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E122" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F122" s="5" t="s">
         <v>15</v>
@@ -4105,10 +4231,10 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C123" s="4" t="n">
         <v>400</v>
@@ -4116,11 +4242,12 @@
       <c r="D123" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E123" s="8" t="s">
-        <v>30</v>
+      <c r="E123" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Concentrada</v>
       </c>
       <c r="F123" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G123" s="6" t="n">
         <v>1</v>
@@ -4129,12 +4256,12 @@
         <v>22</v>
       </c>
       <c r="I123" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B124" s="4" t="s">
         <v>12</v>
@@ -4158,9 +4285,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B125" s="4" t="s">
         <v>17</v>
@@ -4184,9 +4311,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B126" s="4" t="s">
         <v>17</v>
@@ -4209,10 +4336,13 @@
       <c r="H126" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I126" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B127" s="4" t="s">
         <v>17</v>
@@ -4221,10 +4351,10 @@
         <v>250</v>
       </c>
       <c r="D127" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E127" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F127" s="5" t="s">
         <v>15</v>
@@ -4238,10 +4368,10 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C128" s="4" t="n">
         <v>500</v>
@@ -4249,11 +4379,12 @@
       <c r="D128" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E128" s="8" t="s">
-        <v>30</v>
+      <c r="E128" s="10" t="str">
+        <f aca="false">Rotulos[[#This Row],[Concentração]]</f>
+        <v>Fragrância Ultra Concentrada</v>
       </c>
       <c r="F128" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G128" s="6" t="n">
         <v>1</v>
@@ -4262,143 +4393,137 @@
         <v>22</v>
       </c>
       <c r="I128" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="C129" s="4" t="n">
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="D129" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E129" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="F129" s="9" t="s">
-        <v>31</v>
+        <v>13</v>
+      </c>
+      <c r="E129" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F129" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G129" s="6" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="H129" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I129" s="4" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="C130" s="4" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E130" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="F130" s="9" t="s">
-        <v>31</v>
+        <v>18</v>
+      </c>
+      <c r="E130" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F130" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G130" s="6" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="H130" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I130" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="131" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="C131" s="4" t="n">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="D131" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E131" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="F131" s="9" t="s">
-        <v>31</v>
+      <c r="E131" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F131" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G131" s="6" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H131" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="I131" s="4" t="s">
-        <v>33</v>
+      <c r="I131" s="8" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B132" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C132" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="D132" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E132" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F132" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G132" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="H132" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B133" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C132" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="D132" s="4" t="s">
+      <c r="C133" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D133" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E132" s="4" t="s">
+      <c r="E133" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F132" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G132" s="6" t="n">
+      <c r="F133" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G133" s="6" t="n">
         <v>200</v>
-      </c>
-      <c r="H132" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A133" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B133" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C133" s="4" t="n">
-        <v>250</v>
-      </c>
-      <c r="D133" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E133" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F133" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G133" s="6" t="n">
-        <v>18</v>
       </c>
       <c r="H133" s="7" t="s">
         <v>16</v>
@@ -4406,7 +4531,7 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B134" s="4" t="s">
         <v>17</v>
@@ -4415,24 +4540,24 @@
         <v>250</v>
       </c>
       <c r="D134" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E134" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F134" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G134" s="6" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H134" s="7" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B135" s="4" t="s">
         <v>17</v>
@@ -4441,68 +4566,71 @@
         <v>250</v>
       </c>
       <c r="D135" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E135" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F135" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G135" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="H135" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I135" s="8" t="s">
         <v>23</v>
-      </c>
-      <c r="E135" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F135" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G135" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="H135" s="7" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B136" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C136" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="D136" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E136" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F136" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G136" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="H136" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B137" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C136" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="D136" s="4" t="s">
+      <c r="C137" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D137" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E136" s="4" t="s">
+      <c r="E137" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F136" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G136" s="6" t="n">
+      <c r="F137" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G137" s="6" t="n">
         <v>200</v>
-      </c>
-      <c r="H136" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B137" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C137" s="4" t="n">
-        <v>250</v>
-      </c>
-      <c r="D137" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E137" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F137" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G137" s="6" t="n">
-        <v>18</v>
       </c>
       <c r="H137" s="7" t="s">
         <v>16</v>
@@ -4510,7 +4638,7 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B138" s="4" t="s">
         <v>17</v>
@@ -4519,24 +4647,24 @@
         <v>250</v>
       </c>
       <c r="D138" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E138" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F138" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G138" s="6" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H138" s="7" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B139" s="4" t="s">
         <v>17</v>
@@ -4545,68 +4673,71 @@
         <v>250</v>
       </c>
       <c r="D139" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E139" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F139" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G139" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="H139" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I139" s="8" t="s">
         <v>23</v>
-      </c>
-      <c r="E139" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F139" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G139" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="H139" s="7" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B140" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C140" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="D140" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E140" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F140" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G140" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="H140" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B141" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C140" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="D140" s="4" t="s">
+      <c r="C141" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D141" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E140" s="4" t="s">
+      <c r="E141" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F140" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G140" s="6" t="n">
+      <c r="F141" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G141" s="6" t="n">
         <v>200</v>
-      </c>
-      <c r="H140" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A141" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B141" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C141" s="4" t="n">
-        <v>250</v>
-      </c>
-      <c r="D141" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E141" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F141" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G141" s="6" t="n">
-        <v>18</v>
       </c>
       <c r="H141" s="7" t="s">
         <v>16</v>
@@ -4614,7 +4745,7 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B142" s="4" t="s">
         <v>17</v>
@@ -4623,24 +4754,24 @@
         <v>250</v>
       </c>
       <c r="D142" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E142" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F142" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G142" s="6" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H142" s="7" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B143" s="4" t="s">
         <v>17</v>
@@ -4649,150 +4780,75 @@
         <v>250</v>
       </c>
       <c r="D143" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E143" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F143" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G143" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="H143" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I143" s="8" t="s">
         <v>23</v>
-      </c>
-      <c r="E143" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F143" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G143" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="H143" s="7" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C144" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="D144" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E144" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F144" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G144" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="H144" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F146" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="G146" s="12" t="n">
+        <f aca="false">SUBTOTAL(9,G5:G144)</f>
+        <v>4642</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F147" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="B144" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C144" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="D144" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E144" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F144" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G144" s="6" t="n">
-        <v>200</v>
-      </c>
-      <c r="H144" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A145" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B145" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C145" s="4" t="n">
-        <v>250</v>
-      </c>
-      <c r="D145" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E145" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F145" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G145" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="H145" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="146" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A146" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B146" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C146" s="4" t="n">
-        <v>250</v>
-      </c>
-      <c r="D146" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E146" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F146" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G146" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="H146" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A147" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B147" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C147" s="4" t="n">
-        <v>250</v>
-      </c>
-      <c r="D147" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E147" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F147" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G147" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="H147" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F149" s="10" t="s">
+      <c r="G147" s="12" t="n">
+        <f aca="false">SUMIFS(G5:G144,F5:F144,"B2C")</f>
+        <v>4436</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F148" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="G149" s="11" t="n">
-        <f aca="false">SUBTOTAL(9,G5:G147)</f>
-        <v>4647</v>
-      </c>
-    </row>
-    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F150" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="G150" s="11" t="n">
-        <f aca="false">SUMIFS(G5:G147,F5:F147,"B2C")</f>
-        <v>4436</v>
-      </c>
-    </row>
-    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F151" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="G151" s="11" t="n">
-        <f aca="false">SUMIFS(G5:G147,F5:F147,"B2B")</f>
-        <v>211</v>
+      <c r="G148" s="12" t="n">
+        <f aca="false">SUMIFS(G5:G144,F5:F144,"B2B")</f>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -4815,7 +4871,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
@@ -4824,345 +4880,345 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
+      <c r="E4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="12" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="E4" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="13" t="n">
-        <v>15</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="D5" s="13" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$147,$A5,Rótulos!$C$5:$C$147,$B5,Rótulos!$I$5:$I$147,"")</f>
+      <c r="D5" s="8" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$144,$A5,Rótulos!$C$5:$C$144,$B5,Rótulos!$I$5:$I$144,"")</f>
         <v>24</v>
       </c>
-      <c r="E5" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A5,Rótulos!$C$5:$C$147,$B5,Rótulos!$I$5:$I$147,"",Rótulos!$F$5:$F$147,"B2C")</f>
+      <c r="E5" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A5,Rótulos!$C$5:$C$144,$B5,Rótulos!$I$5:$I$144,"",Rótulos!$F$5:$F$144,"B2C")</f>
         <v>3400</v>
       </c>
-      <c r="F5" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A5,Rótulos!$C$5:$C$147,$B5,Rótulos!$I$5:$I$147,"",Rótulos!$F$5:$F$147,"B2B")</f>
+      <c r="F5" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A5,Rótulos!$C$5:$C$144,$B5,Rótulos!$I$5:$I$144,"",Rótulos!$F$5:$F$144,"B2B")</f>
         <v>0</v>
       </c>
-      <c r="G5" s="13" t="n">
+      <c r="G5" s="8" t="n">
         <f aca="false">E5+F5</f>
         <v>3400</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="13" t="n">
-        <v>250</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="D6" s="13" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$147,$A6,Rótulos!$C$5:$C$147,$B6,Rótulos!$I$5:$I$147,"")</f>
+      <c r="A6" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>250</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$144,$A6,Rótulos!$C$5:$C$144,$B6,Rótulos!$I$5:$I$144,"")</f>
         <v>34</v>
       </c>
-      <c r="E6" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A6,Rótulos!$C$5:$C$147,$B6,Rótulos!$I$5:$I$147,"",Rótulos!$F$5:$F$147,"B2C")</f>
+      <c r="E6" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A6,Rótulos!$C$5:$C$144,$B6,Rótulos!$I$5:$I$144,"",Rótulos!$F$5:$F$144,"B2C")</f>
         <v>472</v>
       </c>
-      <c r="F6" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A6,Rótulos!$C$5:$C$147,$B6,Rótulos!$I$5:$I$147,"",Rótulos!$F$5:$F$147,"B2B")</f>
+      <c r="F6" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A6,Rótulos!$C$5:$C$144,$B6,Rótulos!$I$5:$I$144,"",Rótulos!$F$5:$F$144,"B2B")</f>
         <v>0</v>
       </c>
-      <c r="G6" s="13" t="n">
+      <c r="G6" s="8" t="n">
         <f aca="false">E6+F6</f>
         <v>472</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="13" t="n">
+      <c r="A7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="C7" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="13" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$147,$A7,Rótulos!$C$5:$C$147,$B7,Rótulos!$I$5:$I$147,$C7)</f>
-        <v>11</v>
-      </c>
-      <c r="E7" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A7,Rótulos!$C$5:$C$147,$B7,Rótulos!$I$5:$I$147,$C7,Rótulos!$F$5:$F$147,"B2C")</f>
+      <c r="C7" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$144,$A7,Rótulos!$C$5:$C$144,$B7,Rótulos!$I$5:$I$144,$C7)</f>
+        <v>19</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A7,Rótulos!$C$5:$C$144,$B7,Rótulos!$I$5:$I$144,$C7,Rótulos!$F$5:$F$144,"B2C")</f>
+        <v>360</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A7,Rótulos!$C$5:$C$144,$B7,Rótulos!$I$5:$I$144,$C7,Rótulos!$F$5:$F$144,"B2B")</f>
+        <v>88</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <f aca="false">E7+F7</f>
+        <v>448</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$144,$A8,Rótulos!$C$5:$C$144,$B8,Rótulos!$I$5:$I$144,"")</f>
         <v>0</v>
       </c>
-      <c r="F7" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A7,Rótulos!$C$5:$C$147,$B7,Rótulos!$I$5:$I$147,$C7,Rótulos!$F$5:$F$147,"B2B")</f>
-        <v>88</v>
-      </c>
-      <c r="G7" s="13" t="n">
-        <f aca="false">E7+F7</f>
-        <v>88</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="D8" s="13" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$147,$A8,Rótulos!$C$5:$C$147,$B8,Rótulos!$I$5:$I$147,"")</f>
-        <v>8</v>
-      </c>
-      <c r="E8" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A8,Rótulos!$C$5:$C$147,$B8,Rótulos!$I$5:$I$147,"",Rótulos!$F$5:$F$147,"B2C")</f>
-        <v>360</v>
-      </c>
-      <c r="F8" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A8,Rótulos!$C$5:$C$147,$B8,Rótulos!$I$5:$I$147,"",Rótulos!$F$5:$F$147,"B2B")</f>
+      <c r="E8" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A8,Rótulos!$C$5:$C$144,$B8,Rótulos!$I$5:$I$144,"",Rótulos!$F$5:$F$144,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="G8" s="13" t="n">
+      <c r="F8" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A8,Rótulos!$C$5:$C$144,$B8,Rótulos!$I$5:$I$144,"",Rótulos!$F$5:$F$144,"B2B")</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="8" t="n">
         <f aca="false">E8+F8</f>
-        <v>360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="13" t="n">
+      <c r="A9" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="C9" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="D9" s="13" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$147,$A9,Rótulos!$C$5:$C$147,$B9,Rótulos!$I$5:$I$147,$C9)</f>
+      <c r="C9" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$144,$A9,Rótulos!$C$5:$C$144,$B9,Rótulos!$I$5:$I$144,$C9)</f>
         <v>2</v>
       </c>
-      <c r="E9" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A9,Rótulos!$C$5:$C$147,$B9,Rótulos!$I$5:$I$147,$C9,Rótulos!$F$5:$F$147,"B2C")</f>
+      <c r="E9" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A9,Rótulos!$C$5:$C$144,$B9,Rótulos!$I$5:$I$144,$C9,Rótulos!$F$5:$F$144,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="F9" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A9,Rótulos!$C$5:$C$147,$B9,Rótulos!$I$5:$I$147,$C9,Rótulos!$F$5:$F$147,"B2B")</f>
+      <c r="F9" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A9,Rótulos!$C$5:$C$144,$B9,Rótulos!$I$5:$I$144,$C9,Rótulos!$F$5:$F$144,"B2B")</f>
         <v>4</v>
       </c>
-      <c r="G9" s="13" t="n">
+      <c r="G9" s="8" t="n">
         <f aca="false">E9+F9</f>
         <v>4</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="13" t="n">
-        <v>250</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="D10" s="13" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$147,$A10,Rótulos!$C$5:$C$147,$B10,Rótulos!$I$5:$I$147,$C10)</f>
-        <v>4</v>
-      </c>
-      <c r="E10" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A10,Rótulos!$C$5:$C$147,$B10,Rótulos!$I$5:$I$147,$C10,Rótulos!$F$5:$F$147,"B2C")</f>
+      <c r="A10" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>250</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$144,$A10,Rótulos!$C$5:$C$144,$B10,Rótulos!$I$5:$I$144,$C10)</f>
+        <v>21</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A10,Rótulos!$C$5:$C$144,$B10,Rótulos!$I$5:$I$144,$C10,Rótulos!$F$5:$F$144,"B2C")</f>
+        <v>134</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A10,Rótulos!$C$5:$C$144,$B10,Rótulos!$I$5:$I$144,$C10,Rótulos!$F$5:$F$144,"B2B")</f>
+        <v>20</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <f aca="false">E10+F10</f>
+        <v>154</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>250</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$144,$A11,Rótulos!$C$5:$C$144,$B11,Rótulos!$I$5:$I$144,"")</f>
         <v>0</v>
       </c>
-      <c r="F10" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A10,Rótulos!$C$5:$C$147,$B10,Rótulos!$I$5:$I$147,$C10,Rótulos!$F$5:$F$147,"B2B")</f>
-        <v>20</v>
-      </c>
-      <c r="G10" s="13" t="n">
-        <f aca="false">E10+F10</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="13" t="n">
-        <v>250</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="D11" s="13" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$147,$A11,Rótulos!$C$5:$C$147,$B11,Rótulos!$I$5:$I$147,"")</f>
-        <v>17</v>
-      </c>
-      <c r="E11" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A11,Rótulos!$C$5:$C$147,$B11,Rótulos!$I$5:$I$147,"",Rótulos!$F$5:$F$147,"B2C")</f>
-        <v>134</v>
-      </c>
-      <c r="F11" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A11,Rótulos!$C$5:$C$147,$B11,Rótulos!$I$5:$I$147,"",Rótulos!$F$5:$F$147,"B2B")</f>
+      <c r="E11" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A11,Rótulos!$C$5:$C$144,$B11,Rótulos!$I$5:$I$144,"",Rótulos!$F$5:$F$144,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="G11" s="13" t="n">
+      <c r="F11" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A11,Rótulos!$C$5:$C$144,$B11,Rótulos!$I$5:$I$144,"",Rótulos!$F$5:$F$144,"B2B")</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="8" t="n">
         <f aca="false">E11+F11</f>
-        <v>134</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="13" t="n">
+      <c r="A12" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="C12" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="13" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$147,$A12,Rótulos!$C$5:$C$147,$B12,Rótulos!$I$5:$I$147,$C12)</f>
-        <v>12</v>
-      </c>
-      <c r="E12" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A12,Rótulos!$C$5:$C$147,$B12,Rótulos!$I$5:$I$147,$C12,Rótulos!$F$5:$F$147,"B2C")</f>
+      <c r="C12" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$144,$A12,Rótulos!$C$5:$C$144,$B12,Rótulos!$I$5:$I$144,$C12)</f>
+        <v>11</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A12,Rótulos!$C$5:$C$144,$B12,Rótulos!$I$5:$I$144,$C12,Rótulos!$F$5:$F$144,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="F12" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A12,Rótulos!$C$5:$C$147,$B12,Rótulos!$I$5:$I$147,$C12,Rótulos!$F$5:$F$147,"B2B")</f>
-        <v>39</v>
-      </c>
-      <c r="G12" s="13" t="n">
+      <c r="F12" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A12,Rótulos!$C$5:$C$144,$B12,Rótulos!$I$5:$I$144,$C12,Rótulos!$F$5:$F$144,"B2B")</f>
+        <v>37</v>
+      </c>
+      <c r="G12" s="8" t="n">
         <f aca="false">E12+F12</f>
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="13" t="n">
+      <c r="A13" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="8" t="n">
         <v>500</v>
       </c>
-      <c r="C13" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="13" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$147,$A13,Rótulos!$C$5:$C$147,$B13,Rótulos!$I$5:$I$147,$C13)</f>
-        <v>10</v>
-      </c>
-      <c r="E13" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A13,Rótulos!$C$5:$C$147,$B13,Rótulos!$I$5:$I$147,$C13,Rótulos!$F$5:$F$147,"B2C")</f>
+      <c r="C13" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$144,$A13,Rótulos!$C$5:$C$144,$B13,Rótulos!$I$5:$I$144,$C13)</f>
+        <v>16</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A13,Rótulos!$C$5:$C$144,$B13,Rótulos!$I$5:$I$144,$C13,Rótulos!$F$5:$F$144,"B2C")</f>
+        <v>70</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A13,Rótulos!$C$5:$C$144,$B13,Rótulos!$I$5:$I$144,$C13,Rótulos!$F$5:$F$144,"B2B")</f>
+        <v>31</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <f aca="false">E13+F13</f>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$144,$A14,Rótulos!$C$5:$C$144,$B14,Rótulos!$I$5:$I$144,"")</f>
         <v>0</v>
       </c>
-      <c r="F13" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A13,Rótulos!$C$5:$C$147,$B13,Rótulos!$I$5:$I$147,$C13,Rótulos!$F$5:$F$147,"B2B")</f>
-        <v>33</v>
-      </c>
-      <c r="G13" s="13" t="n">
-        <f aca="false">E13+F13</f>
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" s="13" t="n">
-        <v>500</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="D14" s="13" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$147,$A14,Rótulos!$C$5:$C$147,$B14,Rótulos!$I$5:$I$147,"")</f>
-        <v>7</v>
-      </c>
-      <c r="E14" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A14,Rótulos!$C$5:$C$147,$B14,Rótulos!$I$5:$I$147,"",Rótulos!$F$5:$F$147,"B2C")</f>
-        <v>70</v>
-      </c>
-      <c r="F14" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A14,Rótulos!$C$5:$C$147,$B14,Rótulos!$I$5:$I$147,"",Rótulos!$F$5:$F$147,"B2B")</f>
+      <c r="E14" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A14,Rótulos!$C$5:$C$144,$B14,Rótulos!$I$5:$I$144,"",Rótulos!$F$5:$F$144,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="G14" s="13" t="n">
+      <c r="F14" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A14,Rótulos!$C$5:$C$144,$B14,Rótulos!$I$5:$I$144,"",Rótulos!$F$5:$F$144,"B2B")</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="8" t="n">
         <f aca="false">E14+F14</f>
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B15" s="13" t="n">
+      <c r="A15" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="8" t="n">
         <v>1000</v>
       </c>
-      <c r="C15" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="13" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$147,$A15,Rótulos!$C$5:$C$147,$B15,Rótulos!$I$5:$I$147,$C15)</f>
-        <v>14</v>
-      </c>
-      <c r="E15" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A15,Rótulos!$C$5:$C$147,$B15,Rótulos!$I$5:$I$147,$C15,Rótulos!$F$5:$F$147,"B2C")</f>
+      <c r="C15" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$144,$A15,Rótulos!$C$5:$C$144,$B15,Rótulos!$I$5:$I$144,$C15)</f>
+        <v>13</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A15,Rótulos!$C$5:$C$144,$B15,Rótulos!$I$5:$I$144,$C15,Rótulos!$F$5:$F$144,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="F15" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A15,Rótulos!$C$5:$C$147,$B15,Rótulos!$I$5:$I$147,$C15,Rótulos!$F$5:$F$147,"B2B")</f>
-        <v>27</v>
-      </c>
-      <c r="G15" s="13" t="n">
+      <c r="F15" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A15,Rótulos!$C$5:$C$144,$B15,Rótulos!$I$5:$I$144,$C15,Rótulos!$F$5:$F$144,"B2B")</f>
+        <v>26</v>
+      </c>
+      <c r="G15" s="8" t="n">
         <f aca="false">E15+F15</f>
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="14"/>
       <c r="D16" s="14" t="n">
         <f aca="false">SUM(D5:D15)</f>
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E16" s="14" t="n">
         <f aca="false">SUM(E5:E15)</f>
@@ -5170,84 +5226,84 @@
       </c>
       <c r="F16" s="14" t="n">
         <f aca="false">SUM(F5:F15)</f>
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="G16" s="14" t="n">
         <f aca="false">SUM(G5:G15)</f>
-        <v>4647</v>
+        <v>4642</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
-        <v>83</v>
+      <c r="A18" s="11" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E19" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="B19" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="E19" s="15" t="s">
-        <v>81</v>
-      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B20" s="13" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$147,$A20)</f>
+      <c r="A20" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="8" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$144,$A20)</f>
         <v>58</v>
       </c>
-      <c r="C20" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A20,Rótulos!$F$5:$F$147,"B2C")</f>
+      <c r="C20" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A20,Rótulos!$F$5:$F$144,"B2C")</f>
         <v>3872</v>
       </c>
-      <c r="D20" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A20,Rótulos!$F$5:$F$147,"B2B")</f>
+      <c r="D20" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A20,Rótulos!$F$5:$F$144,"B2B")</f>
         <v>0</v>
       </c>
-      <c r="E20" s="13" t="n">
+      <c r="E20" s="8" t="n">
         <f aca="false">C20+D20</f>
         <v>3872</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="13" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$147,$A21)</f>
-        <v>85</v>
-      </c>
-      <c r="C21" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A21,Rótulos!$F$5:$F$147,"B2C")</f>
+      <c r="A21" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="8" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$144,$A21)</f>
+        <v>82</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A21,Rótulos!$F$5:$F$144,"B2C")</f>
         <v>564</v>
       </c>
-      <c r="D21" s="13" t="n">
-        <f aca="false">SUMIFS(Rótulos!$G$5:$G$147,Rótulos!$H$5:$H$147,$A21,Rótulos!$F$5:$F$147,"B2B")</f>
-        <v>211</v>
-      </c>
-      <c r="E21" s="13" t="n">
+      <c r="D21" s="8" t="n">
+        <f aca="false">SUMIFS(Rótulos!$G$5:$G$144,Rótulos!$H$5:$H$144,$A21,Rótulos!$F$5:$F$144,"B2B")</f>
+        <v>206</v>
+      </c>
+      <c r="E21" s="8" t="n">
         <f aca="false">C21+D21</f>
-        <v>775</v>
+        <v>770</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B22" s="14" t="n">
         <f aca="false">SUM(B20:B21)</f>
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C22" s="14" t="n">
         <f aca="false">SUM(C20:C21)</f>
@@ -5255,11 +5311,11 @@
       </c>
       <c r="D22" s="14" t="n">
         <f aca="false">SUM(D20:D21)</f>
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="E22" s="14" t="n">
         <f aca="false">SUM(E20:E21)</f>
-        <v>4647</v>
+        <v>4642</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adiciona aba de versões de rótulo para orçamento
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018k4AWMEfPQ3PeJhEoKFmKz
</commit_message>
<xml_diff>
--- a/Rotulos_Consolidado_atualizado.xlsx
+++ b/Rotulos_Consolidado_atualizado.xlsx
@@ -9,9 +9,10 @@
   </bookViews>
   <sheets>
     <sheet name="Rótulos" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Por Fragrância" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Resumo por Tipo" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="B2B Antes x Depois" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Versões para Orçamento" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Por Fragrância" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Resumo por Tipo" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="B2B Antes x Depois" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2905" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2985" uniqueCount="135">
   <si>
     <t xml:space="preserve">Necessidade de rótulos – consolidado</t>
   </si>
@@ -310,6 +311,54 @@
     <t xml:space="preserve">Total B2B</t>
   </si>
   <si>
+    <t xml:space="preserve">Versões de rótulo para orçamento – por material, tamanho e canal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Versão = arte única (fragrância × concentração × volume) no mesmo material e tamanho. Fórmulas sobre as abas Por Fragrância e Rótulos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Material / tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nº de versões (artes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qtd. total de rótulos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menor tiragem por versão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maior tiragem por versão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Média por versão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nº versões se separar formato e canal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B2B e B2C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A definir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resumo por material e tamanho (todos os canais)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Nº versões se separar formato e canal": conta cada linha da aba Rótulos como arte própria (ex.: Válvula Spray e Kit Varetas com artes diferentes; mesmo rótulo B2B e B2C com artes diferentes). Linhas "B2B e B2C" mostram "-" nessa coluna porque já estão contadas nas linhas B2B e B2C.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rótulo 5 x 10 cm (frente e verso): quantidade = nº de frascos; se forem 2 rótulos por frasco, dobrar no orçamento.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Quantidades por fragrância × concentração × volume</t>
   </si>
   <si>
@@ -317,9 +366,6 @@
   </si>
   <si>
     <t xml:space="preserve">Formatos agrupados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Canal</t>
   </si>
   <si>
     <t xml:space="preserve">Qtd. B2C</t>
@@ -335,9 +381,6 @@
   </si>
   <si>
     <t xml:space="preserve">Perfume para Ambientes + Perfume de Ambientes – Refil PET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B2B e B2C</t>
   </si>
   <si>
     <t xml:space="preserve">Aromatizador de Ambientes + Aromatizador (Refil)</t>
@@ -356,12 +399,6 @@
   </si>
   <si>
     <t xml:space="preserve">Nº linhas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A definir</t>
   </si>
   <si>
     <t xml:space="preserve">Por tamanho (todos os tipos)</t>
@@ -398,10 +435,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0;\-#,##0;\-"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -559,7 +597,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -612,6 +650,22 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -621,14 +675,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -7101,6 +7147,670 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="12" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A5,'Por Fragrância'!$E$5:$E$192,$B5,'Por Fragrância'!$G$5:$G$192,$C5)</f>
+        <v>17</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A5,'Por Fragrância'!$E$5:$E$192,$B5,'Por Fragrância'!$G$5:$G$192,$C5)</f>
+        <v>472</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <f aca="false">_xlfn.MINIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A5,'Por Fragrância'!$E$5:$E$192,$B5,'Por Fragrância'!$G$5:$G$192,$C5)</f>
+        <v>16</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <f aca="false">_xlfn.MAXIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A5,'Por Fragrância'!$E$5:$E$192,$B5,'Por Fragrância'!$G$5:$G$192,$C5)</f>
+        <v>36</v>
+      </c>
+      <c r="H5" s="13" t="n">
+        <f aca="false">IF(D5=0,0,E5/D5)</f>
+        <v>27.7647058823529</v>
+      </c>
+      <c r="I5" s="11" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A5,Rótulos!$I$5:$I$212,$B5,Rótulos!$F$5:$F$212,IF($C5="B2B e B2C","~",$C5))</f>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="12" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A6,'Por Fragrância'!$E$5:$E$192,$B6,'Por Fragrância'!$G$5:$G$192,$C6)</f>
+        <v>24</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A6,'Por Fragrância'!$E$5:$E$192,$B6,'Por Fragrância'!$G$5:$G$192,$C6)</f>
+        <v>3400</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <f aca="false">_xlfn.MINIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A6,'Por Fragrância'!$E$5:$E$192,$B6,'Por Fragrância'!$G$5:$G$192,$C6)</f>
+        <v>100</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <f aca="false">_xlfn.MAXIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A6,'Por Fragrância'!$E$5:$E$192,$B6,'Por Fragrância'!$G$5:$G$192,$C6)</f>
+        <v>200</v>
+      </c>
+      <c r="H6" s="13" t="n">
+        <f aca="false">IF(D6=0,0,E6/D6)</f>
+        <v>141.666666666667</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A6,Rótulos!$I$5:$I$212,$B6,Rótulos!$F$5:$F$212,IF($C6="B2B e B2C","~",$C6))</f>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A7,'Por Fragrância'!$E$5:$E$192,$B7,'Por Fragrância'!$G$5:$G$192,$C7)</f>
+        <v>23</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A7,'Por Fragrância'!$E$5:$E$192,$B7,'Por Fragrância'!$G$5:$G$192,$C7)</f>
+        <v>1307</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <f aca="false">_xlfn.MINIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A7,'Por Fragrância'!$E$5:$E$192,$B7,'Por Fragrância'!$G$5:$G$192,$C7)</f>
+        <v>2</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <f aca="false">_xlfn.MAXIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A7,'Por Fragrância'!$E$5:$E$192,$B7,'Por Fragrância'!$G$5:$G$192,$C7)</f>
+        <v>649</v>
+      </c>
+      <c r="H7" s="13" t="n">
+        <f aca="false">IF(D7=0,0,E7/D7)</f>
+        <v>56.8260869565217</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A7,Rótulos!$I$5:$I$212,$B7,Rótulos!$F$5:$F$212,IF($C7="B2B e B2C","~",$C7))</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A8,'Por Fragrância'!$E$5:$E$192,$B8,'Por Fragrância'!$G$5:$G$192,$C8)</f>
+        <v>8</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A8,'Por Fragrância'!$E$5:$E$192,$B8,'Por Fragrância'!$G$5:$G$192,$C8)</f>
+        <v>360</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <f aca="false">_xlfn.MINIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A8,'Por Fragrância'!$E$5:$E$192,$B8,'Por Fragrância'!$G$5:$G$192,$C8)</f>
+        <v>30</v>
+      </c>
+      <c r="G8" s="11" t="n">
+        <f aca="false">_xlfn.MAXIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A8,'Por Fragrância'!$E$5:$E$192,$B8,'Por Fragrância'!$G$5:$G$192,$C8)</f>
+        <v>150</v>
+      </c>
+      <c r="H8" s="13" t="n">
+        <f aca="false">IF(D8=0,0,E8/D8)</f>
+        <v>45</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A8,Rótulos!$I$5:$I$212,$B8,Rótulos!$F$5:$F$212,IF($C8="B2B e B2C","~",$C8))</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="12" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A9,'Por Fragrância'!$E$5:$E$192,$B9,'Por Fragrância'!$G$5:$G$192,$C9)</f>
+        <v>11</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A9,'Por Fragrância'!$E$5:$E$192,$B9,'Por Fragrância'!$G$5:$G$192,$C9)</f>
+        <v>481</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <f aca="false">_xlfn.MINIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A9,'Por Fragrância'!$E$5:$E$192,$B9,'Por Fragrância'!$G$5:$G$192,$C9)</f>
+        <v>4</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <f aca="false">_xlfn.MAXIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A9,'Por Fragrância'!$E$5:$E$192,$B9,'Por Fragrância'!$G$5:$G$192,$C9)</f>
+        <v>205</v>
+      </c>
+      <c r="H9" s="13" t="n">
+        <f aca="false">IF(D9=0,0,E9/D9)</f>
+        <v>43.7272727272727</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A9,Rótulos!$I$5:$I$212,$B9,Rótulos!$F$5:$F$212,IF($C9="B2B e B2C","~",$C9))</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D10" s="12" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A10,'Por Fragrância'!$E$5:$E$192,$B10,'Por Fragrância'!$G$5:$G$192,$C10)</f>
+        <v>2</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A10,'Por Fragrância'!$E$5:$E$192,$B10,'Por Fragrância'!$G$5:$G$192,$C10)</f>
+        <v>120</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <f aca="false">_xlfn.MINIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A10,'Por Fragrância'!$E$5:$E$192,$B10,'Por Fragrância'!$G$5:$G$192,$C10)</f>
+        <v>38</v>
+      </c>
+      <c r="G10" s="11" t="n">
+        <f aca="false">_xlfn.MAXIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A10,'Por Fragrância'!$E$5:$E$192,$B10,'Por Fragrância'!$G$5:$G$192,$C10)</f>
+        <v>82</v>
+      </c>
+      <c r="H10" s="13" t="n">
+        <f aca="false">IF(D10=0,0,E10/D10)</f>
+        <v>60</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A10,Rótulos!$I$5:$I$212,$B10,Rótulos!$F$5:$F$212,IF($C10="B2B e B2C","~",$C10))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="12" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A11,'Por Fragrância'!$E$5:$E$192,$B11,'Por Fragrância'!$G$5:$G$192,$C11)</f>
+        <v>15</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A11,'Por Fragrância'!$E$5:$E$192,$B11,'Por Fragrância'!$G$5:$G$192,$C11)</f>
+        <v>130</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <f aca="false">_xlfn.MINIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A11,'Por Fragrância'!$E$5:$E$192,$B11,'Por Fragrância'!$G$5:$G$192,$C11)</f>
+        <v>2</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <f aca="false">_xlfn.MAXIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A11,'Por Fragrância'!$E$5:$E$192,$B11,'Por Fragrância'!$G$5:$G$192,$C11)</f>
+        <v>12</v>
+      </c>
+      <c r="H11" s="13" t="n">
+        <f aca="false">IF(D11=0,0,E11/D11)</f>
+        <v>8.66666666666667</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A11,Rótulos!$I$5:$I$212,$B11,Rótulos!$F$5:$F$212,IF($C11="B2B e B2C","~",$C11))</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="12" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A12,'Por Fragrância'!$E$5:$E$192,$B12,'Por Fragrância'!$G$5:$G$192,$C12)</f>
+        <v>53</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A12,'Por Fragrância'!$E$5:$E$192,$B12,'Por Fragrância'!$G$5:$G$192,$C12)</f>
+        <v>1614</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <f aca="false">_xlfn.MINIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A12,'Por Fragrância'!$E$5:$E$192,$B12,'Por Fragrância'!$G$5:$G$192,$C12)</f>
+        <v>1</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <f aca="false">_xlfn.MAXIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A12,'Por Fragrância'!$E$5:$E$192,$B12,'Por Fragrância'!$G$5:$G$192,$C12)</f>
+        <v>379</v>
+      </c>
+      <c r="H12" s="13" t="n">
+        <f aca="false">IF(D12=0,0,E12/D12)</f>
+        <v>30.4528301886792</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A12,Rótulos!$I$5:$I$212,$B12,Rótulos!$F$5:$F$212,IF($C12="B2B e B2C","~",$C12))</f>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A13,'Por Fragrância'!$E$5:$E$192,$B13,'Por Fragrância'!$G$5:$G$192,$C13)</f>
+        <v>1</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A13,'Por Fragrância'!$E$5:$E$192,$B13,'Por Fragrância'!$G$5:$G$192,$C13)</f>
+        <v>50</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <f aca="false">_xlfn.MINIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A13,'Por Fragrância'!$E$5:$E$192,$B13,'Por Fragrância'!$G$5:$G$192,$C13)</f>
+        <v>50</v>
+      </c>
+      <c r="G13" s="11" t="n">
+        <f aca="false">_xlfn.MAXIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A13,'Por Fragrância'!$E$5:$E$192,$B13,'Por Fragrância'!$G$5:$G$192,$C13)</f>
+        <v>50</v>
+      </c>
+      <c r="H13" s="13" t="n">
+        <f aca="false">IF(D13=0,0,E13/D13)</f>
+        <v>50</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A13,Rótulos!$I$5:$I$212,$B13,Rótulos!$F$5:$F$212,IF($C13="B2B e B2C","~",$C13))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="12" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A14,'Por Fragrância'!$E$5:$E$192,$B14,'Por Fragrância'!$G$5:$G$192,$C14)</f>
+        <v>6</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A14,'Por Fragrância'!$E$5:$E$192,$B14,'Por Fragrância'!$G$5:$G$192,$C14)</f>
+        <v>60</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <f aca="false">_xlfn.MINIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A14,'Por Fragrância'!$E$5:$E$192,$B14,'Por Fragrância'!$G$5:$G$192,$C14)</f>
+        <v>10</v>
+      </c>
+      <c r="G14" s="11" t="n">
+        <f aca="false">_xlfn.MAXIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A14,'Por Fragrância'!$E$5:$E$192,$B14,'Por Fragrância'!$G$5:$G$192,$C14)</f>
+        <v>10</v>
+      </c>
+      <c r="H14" s="13" t="n">
+        <f aca="false">IF(D14=0,0,E14/D14)</f>
+        <v>10</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A14,Rótulos!$I$5:$I$212,$B14,Rótulos!$F$5:$F$212,IF($C14="B2B e B2C","~",$C14))</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A15,'Por Fragrância'!$E$5:$E$192,$B15,'Por Fragrância'!$G$5:$G$192,$C15)</f>
+        <v>18</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A15,'Por Fragrância'!$E$5:$E$192,$B15,'Por Fragrância'!$G$5:$G$192,$C15)</f>
+        <v>197</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <f aca="false">_xlfn.MINIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A15,'Por Fragrância'!$E$5:$E$192,$B15,'Por Fragrância'!$G$5:$G$192,$C15)</f>
+        <v>2</v>
+      </c>
+      <c r="G15" s="11" t="n">
+        <f aca="false">_xlfn.MAXIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A15,'Por Fragrância'!$E$5:$E$192,$B15,'Por Fragrância'!$G$5:$G$192,$C15)</f>
+        <v>22</v>
+      </c>
+      <c r="H15" s="13" t="n">
+        <f aca="false">IF(D15=0,0,E15/D15)</f>
+        <v>10.9444444444444</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A15,Rótulos!$I$5:$I$212,$B15,Rótulos!$F$5:$F$212,IF($C15="B2B e B2C","~",$C15))</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A16,'Por Fragrância'!$E$5:$E$192,$B16,'Por Fragrância'!$G$5:$G$192,$C16)</f>
+        <v>10</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A16,'Por Fragrância'!$E$5:$E$192,$B16,'Por Fragrância'!$G$5:$G$192,$C16)</f>
+        <v>141</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <f aca="false">_xlfn.MINIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A16,'Por Fragrância'!$E$5:$E$192,$B16,'Por Fragrância'!$G$5:$G$192,$C16)</f>
+        <v>2</v>
+      </c>
+      <c r="G16" s="11" t="n">
+        <f aca="false">_xlfn.MAXIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A16,'Por Fragrância'!$E$5:$E$192,$B16,'Por Fragrância'!$G$5:$G$192,$C16)</f>
+        <v>29</v>
+      </c>
+      <c r="H16" s="13" t="n">
+        <f aca="false">IF(D16=0,0,E16/D16)</f>
+        <v>14.1</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <f aca="false">SUMPRODUCT((Rótulos!$H$5:$H$212=$A16)*(Rótulos!$I$5:$I$212="")*(Rótulos!$F$5:$F$212=IF($C16="B2B e B2C","~",$C16)))</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12" t="n">
+        <f aca="false">SUM(D5:D16)</f>
+        <v>188</v>
+      </c>
+      <c r="E17" s="12" t="n">
+        <f aca="false">SUM(E5:E16)</f>
+        <v>8332</v>
+      </c>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="12" t="n">
+        <f aca="false">COUNTA(Rótulos!$A$5:$A$212)</f>
+        <v>208</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="16" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A21,'Por Fragrância'!$E$5:$E$192,$B21)</f>
+        <v>17</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A21,'Por Fragrância'!$E$5:$E$192,$B21)</f>
+        <v>472</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="16" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A22,'Por Fragrância'!$E$5:$E$192,$B22)</f>
+        <v>24</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A22,'Por Fragrância'!$E$5:$E$192,$B22)</f>
+        <v>3400</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C23" s="16" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A23,'Por Fragrância'!$E$5:$E$192,$B23)</f>
+        <v>31</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A23,'Por Fragrância'!$E$5:$E$192,$B23)</f>
+        <v>1667</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" s="16" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A24,'Por Fragrância'!$E$5:$E$192,$B24)</f>
+        <v>28</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A24,'Por Fragrância'!$E$5:$E$192,$B24)</f>
+        <v>731</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" s="16" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A25,'Por Fragrância'!$E$5:$E$192,$B25)</f>
+        <v>60</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A25,'Por Fragrância'!$E$5:$E$192,$B25)</f>
+        <v>1724</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" s="16" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A26,'Por Fragrância'!$E$5:$E$192,$B26)</f>
+        <v>18</v>
+      </c>
+      <c r="D26" s="15" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A26,'Por Fragrância'!$E$5:$E$192,$B26)</f>
+        <v>197</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="C27" s="16" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A27,'Por Fragrância'!$E$5:$E$192,$B27)</f>
+        <v>10</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$D$5:$D$192,$A27,'Por Fragrância'!$E$5:$E$192,$B27)</f>
+        <v>141</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16" t="n">
+        <f aca="false">SUM(C21:C27)</f>
+        <v>188</v>
+      </c>
+      <c r="D28" s="16" t="n">
+        <f aca="false">SUM(D21:D27)</f>
+        <v>8332</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:J195"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -7117,12 +7827,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>96</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7142,19 +7852,19 @@
         <v>10</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>98</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7209,7 +7919,7 @@
         <v>21</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>15</v>
@@ -7275,7 +7985,9 @@
       <c r="D8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="4"/>
+      <c r="E8" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="F8" s="4" t="s">
         <v>29</v>
       </c>
@@ -7378,7 +8090,9 @@
       <c r="D11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="4"/>
+      <c r="E11" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="F11" s="4" t="s">
         <v>29</v>
       </c>
@@ -7625,7 +8339,7 @@
         <v>21</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>15</v>
@@ -7761,7 +8475,9 @@
       <c r="D22" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E22" s="4"/>
+      <c r="E22" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="F22" s="4" t="s">
         <v>29</v>
       </c>
@@ -7957,36 +8673,36 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B28" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="C28" s="13" t="n">
+      <c r="B28" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="17" t="n">
         <v>250</v>
       </c>
-      <c r="D28" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="E28" s="13" t="s">
+      <c r="D28" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="E28" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="F28" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="G28" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="H28" s="14" t="n">
+      <c r="F28" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="G28" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="H28" s="18" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$A$5:$A$212,$A28,Rótulos!$B$5:$B$212,$B28,Rótulos!$C$5:$C$212,$C28,Rótulos!$H$5:$H$212,$D28,Rótulos!$I$5:$I$212,$E28,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>2</v>
       </c>
-      <c r="I28" s="14" t="n">
+      <c r="I28" s="18" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$A$5:$A$212,$A28,Rótulos!$B$5:$B$212,$B28,Rótulos!$C$5:$C$212,$C28,Rótulos!$H$5:$H$212,$D28,Rótulos!$I$5:$I$212,$E28,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>36</v>
       </c>
-      <c r="J28" s="15" t="n">
+      <c r="J28" s="19" t="n">
         <f aca="false">H28+I28</f>
         <v>38</v>
       </c>
@@ -8148,7 +8864,7 @@
         <v>21</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G33" s="4" t="s">
         <v>15</v>
@@ -8272,36 +8988,36 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="13" t="s">
+      <c r="A37" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="B37" s="13" t="s">
+      <c r="B37" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C37" s="13" t="n">
+      <c r="C37" s="17" t="n">
         <v>500</v>
       </c>
-      <c r="D37" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="E37" s="13" t="s">
+      <c r="D37" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="E37" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="F37" s="13" t="s">
+      <c r="F37" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="G37" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="G37" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="H37" s="14" t="n">
+      <c r="H37" s="18" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$A$5:$A$212,$A37,Rótulos!$B$5:$B$212,$B37,Rótulos!$C$5:$C$212,$C37,Rótulos!$H$5:$H$212,$D37,Rótulos!$I$5:$I$212,$E37,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>10</v>
       </c>
-      <c r="I37" s="14" t="n">
+      <c r="I37" s="18" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$A$5:$A$212,$A37,Rótulos!$B$5:$B$212,$B37,Rótulos!$C$5:$C$212,$C37,Rótulos!$H$5:$H$212,$D37,Rótulos!$I$5:$I$212,$E37,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>40</v>
       </c>
-      <c r="J37" s="15" t="n">
+      <c r="J37" s="19" t="n">
         <f aca="false">H37+I37</f>
         <v>50</v>
       </c>
@@ -8498,7 +9214,7 @@
         <v>21</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G43" s="4" t="s">
         <v>15</v>
@@ -8813,7 +9529,7 @@
         <v>21</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G52" s="4" t="s">
         <v>15</v>
@@ -8949,7 +9665,9 @@
       <c r="D56" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E56" s="4"/>
+      <c r="E56" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="F56" s="4" t="s">
         <v>29</v>
       </c>
@@ -9231,7 +9949,7 @@
         <v>21</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G64" s="4" t="s">
         <v>15</v>
@@ -9425,36 +10143,36 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="13" t="s">
+      <c r="A70" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B70" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="C70" s="13" t="n">
+      <c r="B70" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C70" s="17" t="n">
         <v>250</v>
       </c>
-      <c r="D70" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="E70" s="13" t="s">
+      <c r="D70" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="E70" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="F70" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="G70" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="H70" s="14" t="n">
+      <c r="F70" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="G70" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="H70" s="18" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$A$5:$A$212,$A70,Rótulos!$B$5:$B$212,$B70,Rótulos!$C$5:$C$212,$C70,Rótulos!$H$5:$H$212,$D70,Rótulos!$I$5:$I$212,$E70,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>2</v>
       </c>
-      <c r="I70" s="14" t="n">
+      <c r="I70" s="18" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$A$5:$A$212,$A70,Rótulos!$B$5:$B$212,$B70,Rótulos!$C$5:$C$212,$C70,Rótulos!$H$5:$H$212,$D70,Rótulos!$I$5:$I$212,$E70,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>80</v>
       </c>
-      <c r="J70" s="15" t="n">
+      <c r="J70" s="19" t="n">
         <f aca="false">H70+I70</f>
         <v>82</v>
       </c>
@@ -9616,7 +10334,7 @@
         <v>21</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G75" s="4" t="s">
         <v>15</v>
@@ -9826,7 +10544,7 @@
         <v>21</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G81" s="4" t="s">
         <v>15</v>
@@ -9892,7 +10610,9 @@
       <c r="D83" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E83" s="4"/>
+      <c r="E83" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="F83" s="4" t="s">
         <v>29</v>
       </c>
@@ -10170,7 +10890,9 @@
       <c r="D91" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E91" s="4"/>
+      <c r="E91" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="F91" s="4" t="s">
         <v>29</v>
       </c>
@@ -10308,7 +11030,9 @@
       <c r="D95" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E95" s="4"/>
+      <c r="E95" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="F95" s="4" t="s">
         <v>29</v>
       </c>
@@ -11465,7 +12189,7 @@
         <v>21</v>
       </c>
       <c r="F128" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G128" s="4" t="s">
         <v>15</v>
@@ -11570,7 +12294,7 @@
         <v>21</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G131" s="4" t="s">
         <v>15</v>
@@ -11990,7 +12714,7 @@
         <v>21</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G143" s="4" t="s">
         <v>15</v>
@@ -12126,7 +12850,9 @@
       <c r="D147" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E147" s="4"/>
+      <c r="E147" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="F147" s="4" t="s">
         <v>29</v>
       </c>
@@ -12373,7 +13099,7 @@
         <v>21</v>
       </c>
       <c r="F154" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G154" s="4" t="s">
         <v>15</v>
@@ -12618,7 +13344,7 @@
         <v>21</v>
       </c>
       <c r="F161" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G161" s="4" t="s">
         <v>15</v>
@@ -12754,7 +13480,9 @@
       <c r="D165" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E165" s="4"/>
+      <c r="E165" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="F165" s="4" t="s">
         <v>29</v>
       </c>
@@ -12927,7 +13655,9 @@
       <c r="D170" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E170" s="4"/>
+      <c r="E170" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="F170" s="4" t="s">
         <v>29</v>
       </c>
@@ -13139,7 +13869,7 @@
         <v>21</v>
       </c>
       <c r="F176" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G176" s="4" t="s">
         <v>15</v>
@@ -13384,7 +14114,7 @@
         <v>21</v>
       </c>
       <c r="F183" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G183" s="4" t="s">
         <v>15</v>
@@ -13489,7 +14219,7 @@
         <v>21</v>
       </c>
       <c r="F186" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G186" s="4" t="s">
         <v>15</v>
@@ -13664,7 +14394,7 @@
         <v>21</v>
       </c>
       <c r="F191" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="G191" s="4" t="s">
         <v>15</v>
@@ -13736,7 +14466,7 @@
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="2" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -13753,7 +14483,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -13768,17 +14498,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>4</v>
@@ -13787,7 +14517,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>15</v>
@@ -13796,332 +14526,332 @@
         <v>30</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="16" t="n">
-        <v>15</v>
-      </c>
-      <c r="C5" s="16" t="s">
+      <c r="B5" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="C5" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A5,Rótulos!$C$5:$C$212,$B5,Rótulos!$I$5:$I$212,$C5)</f>
         <v>24</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A5,Rótulos!$C$5:$C$212,$B5,Rótulos!$I$5:$I$212,$C5,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>3400</v>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A5,Rótulos!$C$5:$C$212,$B5,Rótulos!$I$5:$I$212,$C5,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>0</v>
       </c>
-      <c r="G5" s="16" t="n">
+      <c r="G5" s="15" t="n">
         <f aca="false">E5+F5</f>
         <v>3400</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="15" t="n">
         <v>250</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A6,Rótulos!$C$5:$C$212,$B6,Rótulos!$I$5:$I$212,$C6)</f>
         <v>34</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A6,Rótulos!$C$5:$C$212,$B6,Rótulos!$I$5:$I$212,$C6,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>472</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A6,Rótulos!$C$5:$C$212,$B6,Rótulos!$I$5:$I$212,$C6,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>0</v>
       </c>
-      <c r="G6" s="16" t="n">
+      <c r="G6" s="15" t="n">
         <f aca="false">E6+F6</f>
         <v>472</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="16" t="n">
+      <c r="A7" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A7,Rótulos!$C$5:$C$212,$B7,Rótulos!$I$5:$I$212,$C7)</f>
         <v>31</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A7,Rótulos!$C$5:$C$212,$B7,Rótulos!$I$5:$I$212,$C7,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>360</v>
       </c>
-      <c r="F7" s="16" t="n">
+      <c r="F7" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A7,Rótulos!$C$5:$C$212,$B7,Rótulos!$I$5:$I$212,$C7,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>1307</v>
       </c>
-      <c r="G7" s="16" t="n">
+      <c r="G7" s="15" t="n">
         <f aca="false">E7+F7</f>
         <v>1667</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="16" t="n">
+      <c r="A8" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="15" t="n">
         <v>150</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A8,Rótulos!$C$5:$C$212,$B8,Rótulos!$I$5:$I$212,$C8)</f>
         <v>6</v>
       </c>
-      <c r="E8" s="16" t="n">
+      <c r="E8" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A8,Rótulos!$C$5:$C$212,$B8,Rótulos!$I$5:$I$212,$C8,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A8,Rótulos!$C$5:$C$212,$B8,Rótulos!$I$5:$I$212,$C8,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>63</v>
       </c>
-      <c r="G8" s="16" t="n">
+      <c r="G8" s="15" t="n">
         <f aca="false">E8+F8</f>
         <v>63</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="16" t="n">
+      <c r="A9" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="15" t="n">
         <v>160</v>
       </c>
-      <c r="C9" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="D9" s="16" t="n">
+      <c r="C9" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="15" t="n">
         <f aca="false">SUMPRODUCT((Rótulos!$I$5:$I$212="")*(Rótulos!$H$5:$H$212=$A9)*(Rótulos!$C$5:$C$212=$B9))</f>
         <v>6</v>
       </c>
-      <c r="E9" s="16" t="n">
+      <c r="E9" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A9,Rótulos!$C$5:$C$212,$B9,Rótulos!$I$5:$I$212,"=",Rótulos!$F$5:$F$212,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A9,Rótulos!$C$5:$C$212,$B9,Rótulos!$I$5:$I$212,"=",Rótulos!$F$5:$F$212,"B2B")</f>
         <v>95</v>
       </c>
-      <c r="G9" s="16" t="n">
+      <c r="G9" s="15" t="n">
         <f aca="false">E9+F9</f>
         <v>95</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="16" t="n">
+      <c r="A10" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="15" t="n">
         <v>200</v>
       </c>
-      <c r="C10" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="D10" s="16" t="n">
+      <c r="C10" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" s="15" t="n">
         <f aca="false">SUMPRODUCT((Rótulos!$I$5:$I$212="")*(Rótulos!$H$5:$H$212=$A10)*(Rótulos!$C$5:$C$212=$B10))</f>
         <v>1</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A10,Rótulos!$C$5:$C$212,$B10,Rótulos!$I$5:$I$212,"=",Rótulos!$F$5:$F$212,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A10,Rótulos!$C$5:$C$212,$B10,Rótulos!$I$5:$I$212,"=",Rótulos!$F$5:$F$212,"B2B")</f>
         <v>2</v>
       </c>
-      <c r="G10" s="16" t="n">
+      <c r="G10" s="15" t="n">
         <f aca="false">E10+F10</f>
         <v>2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="16" t="n">
+      <c r="A11" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="15" t="n">
         <v>250</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A11,Rótulos!$C$5:$C$212,$B11,Rótulos!$I$5:$I$212,$C11)</f>
         <v>24</v>
       </c>
-      <c r="E11" s="16" t="n">
+      <c r="E11" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A11,Rótulos!$C$5:$C$212,$B11,Rótulos!$I$5:$I$212,$C11,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>134</v>
       </c>
-      <c r="F11" s="16" t="n">
+      <c r="F11" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A11,Rótulos!$C$5:$C$212,$B11,Rótulos!$I$5:$I$212,$C11,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>534</v>
       </c>
-      <c r="G11" s="16" t="n">
+      <c r="G11" s="15" t="n">
         <f aca="false">E11+F11</f>
         <v>668</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="16" t="n">
+      <c r="A12" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="15" t="n">
         <v>400</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A12,Rótulos!$C$5:$C$212,$B12,Rótulos!$I$5:$I$212,$C12)</f>
         <v>26</v>
       </c>
-      <c r="E12" s="16" t="n">
+      <c r="E12" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A12,Rótulos!$C$5:$C$212,$B12,Rótulos!$I$5:$I$212,$C12,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="F12" s="16" t="n">
+      <c r="F12" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A12,Rótulos!$C$5:$C$212,$B12,Rótulos!$I$5:$I$212,$C12,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>635</v>
       </c>
-      <c r="G12" s="16" t="n">
+      <c r="G12" s="15" t="n">
         <f aca="false">E12+F12</f>
         <v>635</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="16" t="n">
+      <c r="A13" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="15" t="n">
         <v>500</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A13,Rótulos!$C$5:$C$212,$B13,Rótulos!$I$5:$I$212,$C13)</f>
         <v>35</v>
       </c>
-      <c r="E13" s="16" t="n">
+      <c r="E13" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A13,Rótulos!$C$5:$C$212,$B13,Rótulos!$I$5:$I$212,$C13,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>70</v>
       </c>
-      <c r="F13" s="16" t="n">
+      <c r="F13" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A13,Rótulos!$C$5:$C$212,$B13,Rótulos!$I$5:$I$212,$C13,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>1019</v>
       </c>
-      <c r="G13" s="16" t="n">
+      <c r="G13" s="15" t="n">
         <f aca="false">E13+F13</f>
         <v>1089</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="16" t="n">
+      <c r="A14" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="15" t="n">
         <v>1000</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="16" t="n">
+      <c r="D14" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A14,Rótulos!$C$5:$C$212,$B14,Rótulos!$I$5:$I$212,$C14)</f>
         <v>18</v>
       </c>
-      <c r="E14" s="16" t="n">
+      <c r="E14" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A14,Rótulos!$C$5:$C$212,$B14,Rótulos!$I$5:$I$212,$C14,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="F14" s="16" t="n">
+      <c r="F14" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A14,Rótulos!$C$5:$C$212,$B14,Rótulos!$I$5:$I$212,$C14,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>197</v>
       </c>
-      <c r="G14" s="16" t="n">
+      <c r="G14" s="15" t="n">
         <f aca="false">E14+F14</f>
         <v>197</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" s="16" t="n">
+      <c r="A15" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="15" t="n">
         <v>5000</v>
       </c>
-      <c r="C15" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="D15" s="16" t="n">
+      <c r="C15" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" s="15" t="n">
         <f aca="false">SUMPRODUCT((Rótulos!$I$5:$I$212="")*(Rótulos!$H$5:$H$212=$A15)*(Rótulos!$C$5:$C$212=$B15))</f>
         <v>3</v>
       </c>
-      <c r="E15" s="16" t="n">
+      <c r="E15" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A15,Rótulos!$C$5:$C$212,$B15,Rótulos!$I$5:$I$212,"=",Rótulos!$F$5:$F$212,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="F15" s="16" t="n">
+      <c r="F15" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A15,Rótulos!$C$5:$C$212,$B15,Rótulos!$I$5:$I$212,"=",Rótulos!$F$5:$F$212,"B2B")</f>
         <v>44</v>
       </c>
-      <c r="G15" s="16" t="n">
+      <c r="G15" s="15" t="n">
         <f aca="false">E15+F15</f>
         <v>44</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
-        <v>111</v>
-      </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17" t="n">
+      <c r="A16" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16" t="n">
         <f aca="false">SUM(D5:D15)</f>
         <v>208</v>
       </c>
-      <c r="E16" s="17" t="n">
+      <c r="E16" s="16" t="n">
         <f aca="false">SUM(E5:E15)</f>
         <v>4436</v>
       </c>
-      <c r="F16" s="17" t="n">
+      <c r="F16" s="16" t="n">
         <f aca="false">SUM(F5:F15)</f>
         <v>3896</v>
       </c>
-      <c r="G16" s="17" t="n">
+      <c r="G16" s="16" t="n">
         <f aca="false">SUM(G5:G15)</f>
         <v>8332</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14129,10 +14859,10 @@
         <v>10</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>15</v>
@@ -14141,195 +14871,195 @@
         <v>30</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="16" t="n">
+      <c r="B20" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$I$5:$I$212,$A20,Rótulos!$H$5:$H$212,$B20)</f>
         <v>31</v>
       </c>
-      <c r="D20" s="16" t="n">
+      <c r="D20" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A20,Rótulos!$H$5:$H$212,$B20,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>360</v>
       </c>
-      <c r="E20" s="16" t="n">
+      <c r="E20" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A20,Rótulos!$H$5:$H$212,$B20,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>1307</v>
       </c>
-      <c r="F20" s="16" t="n">
+      <c r="F20" s="15" t="n">
         <f aca="false">D20+E20</f>
         <v>1667</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="16" t="s">
+      <c r="A21" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C21" s="16" t="n">
+      <c r="B21" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$I$5:$I$212,$A21,Rótulos!$H$5:$H$212,$B21)</f>
         <v>30</v>
       </c>
-      <c r="D21" s="16" t="n">
+      <c r="D21" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A21,Rótulos!$H$5:$H$212,$B21,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>134</v>
       </c>
-      <c r="E21" s="16" t="n">
+      <c r="E21" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A21,Rótulos!$H$5:$H$212,$B21,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>597</v>
       </c>
-      <c r="F21" s="16" t="n">
+      <c r="F21" s="15" t="n">
         <f aca="false">D21+E21</f>
         <v>731</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C22" s="16" t="n">
+      <c r="B22" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$I$5:$I$212,$A22,Rótulos!$H$5:$H$212,$B22)</f>
         <v>61</v>
       </c>
-      <c r="D22" s="16" t="n">
+      <c r="D22" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A22,Rótulos!$H$5:$H$212,$B22,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>70</v>
       </c>
-      <c r="E22" s="16" t="n">
+      <c r="E22" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A22,Rótulos!$H$5:$H$212,$B22,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>1654</v>
       </c>
-      <c r="F22" s="16" t="n">
+      <c r="F22" s="15" t="n">
         <f aca="false">D22+E22</f>
         <v>1724</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="16" t="s">
+      <c r="A23" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C23" s="16" t="n">
+      <c r="B23" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$I$5:$I$212,$A23,Rótulos!$H$5:$H$212,$B23)</f>
         <v>18</v>
       </c>
-      <c r="D23" s="16" t="n">
+      <c r="D23" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A23,Rótulos!$H$5:$H$212,$B23,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="E23" s="16" t="n">
+      <c r="E23" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A23,Rótulos!$H$5:$H$212,$B23,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>197</v>
       </c>
-      <c r="F23" s="16" t="n">
+      <c r="F23" s="15" t="n">
         <f aca="false">D23+E23</f>
         <v>197</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="16" t="s">
+      <c r="B24" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C24" s="16" t="n">
+      <c r="C24" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$I$5:$I$212,$A24,Rótulos!$H$5:$H$212,$B24)</f>
         <v>34</v>
       </c>
-      <c r="D24" s="16" t="n">
+      <c r="D24" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A24,Rótulos!$H$5:$H$212,$B24,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>472</v>
       </c>
-      <c r="E24" s="16" t="n">
+      <c r="E24" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A24,Rótulos!$H$5:$H$212,$B24,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>0</v>
       </c>
-      <c r="F24" s="16" t="n">
+      <c r="F24" s="15" t="n">
         <f aca="false">D24+E24</f>
         <v>472</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="B25" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="16" t="n">
+      <c r="C25" s="15" t="n">
         <f aca="false">COUNTIFS(Rótulos!$I$5:$I$212,$A25,Rótulos!$H$5:$H$212,$B25)</f>
         <v>24</v>
       </c>
-      <c r="D25" s="16" t="n">
+      <c r="D25" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A25,Rótulos!$H$5:$H$212,$B25,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>3400</v>
       </c>
-      <c r="E25" s="16" t="n">
+      <c r="E25" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A25,Rótulos!$H$5:$H$212,$B25,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>0</v>
       </c>
-      <c r="F25" s="16" t="n">
+      <c r="F25" s="15" t="n">
         <f aca="false">D25+E25</f>
         <v>3400</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="B26" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C26" s="16" t="n">
+      <c r="A26" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="C26" s="15" t="n">
         <f aca="false">SUMPRODUCT((Rótulos!$I$5:$I$212="")*(Rótulos!$H$5:$H$212=$B26))</f>
         <v>10</v>
       </c>
-      <c r="D26" s="16" t="n">
+      <c r="D26" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,"=",Rótulos!$H$5:$H$212,$B26,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>0</v>
       </c>
-      <c r="E26" s="16" t="n">
+      <c r="E26" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,"=",Rótulos!$H$5:$H$212,$B26,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>141</v>
       </c>
-      <c r="F26" s="16" t="n">
+      <c r="F26" s="15" t="n">
         <f aca="false">D26+E26</f>
         <v>141</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17" t="s">
-        <v>111</v>
-      </c>
-      <c r="B27" s="17"/>
-      <c r="C27" s="17" t="n">
+      <c r="A27" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="B27" s="16"/>
+      <c r="C27" s="16" t="n">
         <f aca="false">SUM(C20:C26)</f>
         <v>208</v>
       </c>
-      <c r="D27" s="17" t="n">
+      <c r="D27" s="16" t="n">
         <f aca="false">SUM(D20:D26)</f>
         <v>4436</v>
       </c>
-      <c r="E27" s="17" t="n">
+      <c r="E27" s="16" t="n">
         <f aca="false">SUM(E20:E26)</f>
         <v>3896</v>
       </c>
-      <c r="F27" s="17" t="n">
+      <c r="F27" s="16" t="n">
         <f aca="false">SUM(F20:F26)</f>
         <v>8332</v>
       </c>
@@ -14345,7 +15075,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -14362,12 +15092,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14381,13 +15111,13 @@
         <v>4</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14749,7 +15479,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>33</v>
@@ -15379,7 +16109,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>29</v>
@@ -15547,10 +16277,10 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="C60" s="4" t="n">
         <v>500</v>
@@ -17017,7 +17747,7 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="9" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D130" s="10" t="n">
         <f aca="false">SUM(D5:D129)</f>

</xml_diff>

<commit_message>
Troca nº de linhas por nº de versões e adiciona versões por fragrância
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018k4AWMEfPQ3PeJhEoKFmKz
</commit_message>
<xml_diff>
--- a/Rotulos_Consolidado_atualizado.xlsx
+++ b/Rotulos_Consolidado_atualizado.xlsx
@@ -10,10 +10,14 @@
   <sheets>
     <sheet name="Rótulos" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Versões para Orçamento" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Por Fragrância" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Resumo por Tipo" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="B2B Antes x Depois" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Versões por Fragrância" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Por Fragrância" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Resumo por Tipo" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="B2B Antes x Depois" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Versões por Fragrância'!$A$4:$K$60</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -24,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2985" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3111" uniqueCount="145">
   <si>
     <t xml:space="preserve">Necessidade de rótulos – consolidado</t>
   </si>
@@ -359,6 +363,43 @@
     <t xml:space="preserve">Rótulo 5 x 10 cm (frente e verso): quantidade = nº de frascos; se forem 2 rótulos por frasco, dobrar no orçamento.</t>
   </si>
   <si>
+    <t xml:space="preserve">Versões de rótulo por fragrância</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cada número = quantas artes diferentes a fragrância tem naquele material e tamanho (concentrações e volumes distintos). Fórmulas sobre a aba Por Fragrância.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transparente
+5 x 10 cm (frente e verso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transparente
+6,5 x 5 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vinil ou Bopp
+13 x 5 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vinil ou Bopp
+18 x 6,5 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vinil ou Bopp
+22 x 8 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vinil ou Bopp
+28 x 10,5 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vinil ou Bopp
+A definir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total de versões</t>
+  </si>
+  <si>
     <t xml:space="preserve">Quantidades por fragrância × concentração × volume</t>
   </si>
   <si>
@@ -392,13 +433,13 @@
     <t xml:space="preserve">Quantidade de rótulos por tipo, volume e tamanho</t>
   </si>
   <si>
-    <t xml:space="preserve">Fórmulas sobre a aba Rótulos. Tamanho vazio = "A definir".</t>
+    <t xml:space="preserve">Versão = arte única (fragrância × concentração × volume) no mesmo material e tamanho (aba Por Fragrância). Quantidades da aba Rótulos.</t>
   </si>
   <si>
     <t xml:space="preserve">Tipo de rótulo</t>
   </si>
   <si>
-    <t xml:space="preserve">Nº linhas</t>
+    <t xml:space="preserve">Nº de versões de rótulo</t>
   </si>
   <si>
     <t xml:space="preserve">Por tamanho (todos os tipos)</t>
@@ -597,7 +638,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -664,6 +705,14 @@
     </xf>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -805,6 +854,10 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7811,6 +7864,2583 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:K61"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="3" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A5,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D5" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A5,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A5,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A5,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G5" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A5,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A5,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I5" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A5,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="18" t="n">
+        <f aca="false">SUM(C5:I5)</f>
+        <v>3</v>
+      </c>
+      <c r="K5" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A5)</f>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A6,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D6" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A6,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A6,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A6,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G6" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A6,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>3</v>
+      </c>
+      <c r="H6" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A6,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I6" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A6,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>2</v>
+      </c>
+      <c r="J6" s="18" t="n">
+        <f aca="false">SUM(C6:I6)</f>
+        <v>12</v>
+      </c>
+      <c r="K6" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A6)</f>
+        <v>486</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A7,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A7,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A7,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A7,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A7,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H7" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A7,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I7" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A7,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>1</v>
+      </c>
+      <c r="J7" s="18" t="n">
+        <f aca="false">SUM(C7:I7)</f>
+        <v>3</v>
+      </c>
+      <c r="K7" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A7)</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A8,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D8" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A8,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A8,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A8,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A8,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>3</v>
+      </c>
+      <c r="H8" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A8,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="I8" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A8,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J8" s="18" t="n">
+        <f aca="false">SUM(C8:I8)</f>
+        <v>11</v>
+      </c>
+      <c r="K8" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A8)</f>
+        <v>398</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A9,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A9,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A9,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A9,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A9,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A9,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A9,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="18" t="n">
+        <f aca="false">SUM(C9:I9)</f>
+        <v>1</v>
+      </c>
+      <c r="K9" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A9)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A10,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A10,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A10,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A10,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A10,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H10" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A10,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A10,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="18" t="n">
+        <f aca="false">SUM(C10:I10)</f>
+        <v>1</v>
+      </c>
+      <c r="K10" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A10)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C11" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A11,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D11" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A11,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A11,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A11,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="G11" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A11,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H11" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A11,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A11,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="18" t="n">
+        <f aca="false">SUM(C11:I11)</f>
+        <v>9</v>
+      </c>
+      <c r="K11" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A11)</f>
+        <v>365</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A12,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A12,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A12,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A12,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A12,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H12" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A12,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A12,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J12" s="18" t="n">
+        <f aca="false">SUM(C12:I12)</f>
+        <v>1</v>
+      </c>
+      <c r="K12" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A12)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C13" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A13,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D13" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A13,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A13,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A13,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A13,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H13" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A13,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A13,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="18" t="n">
+        <f aca="false">SUM(C13:I13)</f>
+        <v>8</v>
+      </c>
+      <c r="K13" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A13)</f>
+        <v>274</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A14,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A14,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A14,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A14,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G14" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A14,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A14,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I14" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A14,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>1</v>
+      </c>
+      <c r="J14" s="18" t="n">
+        <f aca="false">SUM(C14:I14)</f>
+        <v>3</v>
+      </c>
+      <c r="K14" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A14)</f>
+        <v>231</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A15,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A15,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A15,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A15,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A15,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>3</v>
+      </c>
+      <c r="H15" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A15,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I15" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A15,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="18" t="n">
+        <f aca="false">SUM(C15:I15)</f>
+        <v>5</v>
+      </c>
+      <c r="K15" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A15)</f>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A16,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A16,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A16,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A16,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A16,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H16" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A16,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A16,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J16" s="18" t="n">
+        <f aca="false">SUM(C16:I16)</f>
+        <v>1</v>
+      </c>
+      <c r="K16" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A16)</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A17,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D17" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A17,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="E17" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A17,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A17,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G17" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A17,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A17,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A17,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J17" s="18" t="n">
+        <f aca="false">SUM(C17:I17)</f>
+        <v>3</v>
+      </c>
+      <c r="K17" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A17)</f>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C18" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A18,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D18" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A18,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="E18" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A18,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="F18" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A18,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G18" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A18,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>3</v>
+      </c>
+      <c r="H18" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A18,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I18" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A18,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="18" t="n">
+        <f aca="false">SUM(C18:I18)</f>
+        <v>10</v>
+      </c>
+      <c r="K18" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A18)</f>
+        <v>509</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A19,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A19,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A19,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A19,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G19" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A19,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A19,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I19" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A19,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J19" s="18" t="n">
+        <f aca="false">SUM(C19:I19)</f>
+        <v>1</v>
+      </c>
+      <c r="K19" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A19)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A20,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D20" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A20,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E20" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A20,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A20,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A20,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H20" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A20,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A20,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J20" s="18" t="n">
+        <f aca="false">SUM(C20:I20)</f>
+        <v>1</v>
+      </c>
+      <c r="K20" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A20)</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A21,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A21,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A21,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A21,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A21,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H21" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A21,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A21,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="18" t="n">
+        <f aca="false">SUM(C21:I21)</f>
+        <v>1</v>
+      </c>
+      <c r="K21" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A21)</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A22,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D22" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A22,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E22" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A22,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A22,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A22,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H22" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A22,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I22" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A22,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J22" s="18" t="n">
+        <f aca="false">SUM(C22:I22)</f>
+        <v>1</v>
+      </c>
+      <c r="K22" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A22)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A23,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D23" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A23,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="E23" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A23,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A23,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G23" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A23,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A23,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I23" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A23,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J23" s="18" t="n">
+        <f aca="false">SUM(C23:I23)</f>
+        <v>3</v>
+      </c>
+      <c r="K23" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A23)</f>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C24" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A24,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D24" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A24,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A24,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A24,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G24" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A24,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H24" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A24,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I24" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A24,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>1</v>
+      </c>
+      <c r="J24" s="18" t="n">
+        <f aca="false">SUM(C24:I24)</f>
+        <v>5</v>
+      </c>
+      <c r="K24" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A24)</f>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A25,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A25,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A25,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A25,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A25,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H25" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A25,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A25,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J25" s="18" t="n">
+        <f aca="false">SUM(C25:I25)</f>
+        <v>1</v>
+      </c>
+      <c r="K25" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A25)</f>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A26,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A26,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A26,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A26,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="G26" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A26,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H26" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A26,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A26,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>1</v>
+      </c>
+      <c r="J26" s="18" t="n">
+        <f aca="false">SUM(C26:I26)</f>
+        <v>5</v>
+      </c>
+      <c r="K26" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A26)</f>
+        <v>145</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A27,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A27,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A27,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F27" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A27,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A27,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A27,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I27" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A27,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J27" s="18" t="n">
+        <f aca="false">SUM(C27:I27)</f>
+        <v>1</v>
+      </c>
+      <c r="K27" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A27)</f>
+        <v>649</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A28,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A28,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A28,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F28" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A28,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A28,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H28" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A28,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I28" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A28,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>1</v>
+      </c>
+      <c r="J28" s="18" t="n">
+        <f aca="false">SUM(C28:I28)</f>
+        <v>3</v>
+      </c>
+      <c r="K28" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A28)</f>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A29,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A29,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A29,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F29" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A29,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A29,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H29" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A29,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I29" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A29,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J29" s="18" t="n">
+        <f aca="false">SUM(C29:I29)</f>
+        <v>2</v>
+      </c>
+      <c r="K29" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A29)</f>
+        <v>149</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C30" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A30,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A30,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A30,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F30" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A30,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G30" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A30,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H30" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A30,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="I30" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A30,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J30" s="18" t="n">
+        <f aca="false">SUM(C30:I30)</f>
+        <v>5</v>
+      </c>
+      <c r="K30" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A30)</f>
+        <v>342</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A31,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D31" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A31,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E31" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A31,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A31,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A31,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H31" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A31,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I31" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A31,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J31" s="18" t="n">
+        <f aca="false">SUM(C31:I31)</f>
+        <v>1</v>
+      </c>
+      <c r="K31" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A31)</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A32,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D32" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A32,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E32" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A32,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A32,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G32" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A32,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H32" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A32,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I32" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A32,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J32" s="18" t="n">
+        <f aca="false">SUM(C32:I32)</f>
+        <v>3</v>
+      </c>
+      <c r="K32" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A32)</f>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A33,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D33" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A33,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E33" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A33,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F33" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A33,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G33" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A33,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H33" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A33,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I33" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A33,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J33" s="18" t="n">
+        <f aca="false">SUM(C33:I33)</f>
+        <v>2</v>
+      </c>
+      <c r="K33" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A33)</f>
+        <v>406</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C34" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A34,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D34" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A34,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E34" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A34,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F34" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A34,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G34" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A34,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H34" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A34,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I34" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A34,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J34" s="18" t="n">
+        <f aca="false">SUM(C34:I34)</f>
+        <v>4</v>
+      </c>
+      <c r="K34" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A34)</f>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A35,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D35" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A35,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E35" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A35,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F35" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A35,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G35" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A35,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H35" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A35,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I35" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A35,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J35" s="18" t="n">
+        <f aca="false">SUM(C35:I35)</f>
+        <v>2</v>
+      </c>
+      <c r="K35" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A35)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A36,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D36" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A36,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E36" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A36,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F36" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A36,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G36" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A36,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H36" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A36,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I36" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A36,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J36" s="18" t="n">
+        <f aca="false">SUM(C36:I36)</f>
+        <v>2</v>
+      </c>
+      <c r="K36" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A36)</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A37,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D37" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A37,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E37" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A37,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F37" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A37,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G37" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A37,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H37" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A37,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I37" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A37,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J37" s="18" t="n">
+        <f aca="false">SUM(C37:I37)</f>
+        <v>2</v>
+      </c>
+      <c r="K37" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A37)</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B38" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C38" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A38,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D38" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A38,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A38,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F38" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A38,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G38" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A38,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A38,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I38" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A38,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J38" s="18" t="n">
+        <f aca="false">SUM(C38:I38)</f>
+        <v>1</v>
+      </c>
+      <c r="K38" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A38)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C39" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A39,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D39" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A39,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="E39" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A39,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="F39" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A39,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="G39" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A39,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H39" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A39,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I39" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A39,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J39" s="18" t="n">
+        <f aca="false">SUM(C39:I39)</f>
+        <v>8</v>
+      </c>
+      <c r="K39" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A39)</f>
+        <v>268</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B40" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C40" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A40,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D40" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A40,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="E40" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A40,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F40" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A40,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G40" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A40,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A40,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I40" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A40,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J40" s="18" t="n">
+        <f aca="false">SUM(C40:I40)</f>
+        <v>3</v>
+      </c>
+      <c r="K40" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A40)</f>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C41" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A41,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D41" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A41,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E41" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A41,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F41" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A41,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G41" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A41,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H41" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A41,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I41" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A41,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J41" s="18" t="n">
+        <f aca="false">SUM(C41:I41)</f>
+        <v>1</v>
+      </c>
+      <c r="K41" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A41)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B42" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C42" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A42,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D42" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A42,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E42" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A42,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F42" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A42,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G42" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A42,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H42" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A42,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I42" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A42,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J42" s="18" t="n">
+        <f aca="false">SUM(C42:I42)</f>
+        <v>5</v>
+      </c>
+      <c r="K42" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A42)</f>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="B43" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C43" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A43,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D43" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A43,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="E43" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A43,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F43" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A43,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G43" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A43,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H43" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A43,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I43" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A43,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J43" s="18" t="n">
+        <f aca="false">SUM(C43:I43)</f>
+        <v>6</v>
+      </c>
+      <c r="K43" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A43)</f>
+        <v>258</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C44" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A44,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D44" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A44,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E44" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A44,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F44" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A44,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="G44" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A44,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H44" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A44,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I44" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A44,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>1</v>
+      </c>
+      <c r="J44" s="18" t="n">
+        <f aca="false">SUM(C44:I44)</f>
+        <v>6</v>
+      </c>
+      <c r="K44" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A44)</f>
+        <v>158</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="B45" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C45" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A45,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D45" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A45,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E45" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A45,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F45" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A45,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G45" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A45,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H45" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A45,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I45" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A45,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J45" s="18" t="n">
+        <f aca="false">SUM(C45:I45)</f>
+        <v>1</v>
+      </c>
+      <c r="K45" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A45)</f>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C46" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A46,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A46,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E46" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A46,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F46" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A46,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G46" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A46,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H46" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A46,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I46" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A46,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J46" s="18" t="n">
+        <f aca="false">SUM(C46:I46)</f>
+        <v>1</v>
+      </c>
+      <c r="K46" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A46)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B47" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C47" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A47,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D47" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A47,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="E47" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A47,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F47" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A47,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G47" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A47,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H47" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A47,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I47" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A47,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J47" s="18" t="n">
+        <f aca="false">SUM(C47:I47)</f>
+        <v>3</v>
+      </c>
+      <c r="K47" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A47)</f>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C48" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A48,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D48" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A48,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E48" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A48,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F48" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A48,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G48" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A48,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H48" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A48,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I48" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A48,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J48" s="18" t="n">
+        <f aca="false">SUM(C48:I48)</f>
+        <v>1</v>
+      </c>
+      <c r="K48" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A48)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="B49" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C49" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A49,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D49" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A49,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E49" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A49,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F49" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A49,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G49" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A49,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H49" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A49,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I49" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A49,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J49" s="18" t="n">
+        <f aca="false">SUM(C49:I49)</f>
+        <v>3</v>
+      </c>
+      <c r="K49" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A49)</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C50" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A50,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D50" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A50,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="E50" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A50,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F50" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A50,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G50" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A50,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H50" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A50,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I50" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A50,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J50" s="18" t="n">
+        <f aca="false">SUM(C50:I50)</f>
+        <v>3</v>
+      </c>
+      <c r="K50" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A50)</f>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B51" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C51" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A51,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D51" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A51,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E51" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A51,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F51" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A51,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G51" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A51,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H51" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A51,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I51" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A51,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J51" s="18" t="n">
+        <f aca="false">SUM(C51:I51)</f>
+        <v>2</v>
+      </c>
+      <c r="K51" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A51)</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="B52" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C52" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A52,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D52" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A52,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E52" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A52,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F52" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A52,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G52" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A52,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H52" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A52,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I52" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A52,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>1</v>
+      </c>
+      <c r="J52" s="18" t="n">
+        <f aca="false">SUM(C52:I52)</f>
+        <v>5</v>
+      </c>
+      <c r="K52" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A52)</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B53" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C53" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A53,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D53" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A53,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E53" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A53,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F53" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A53,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G53" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A53,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H53" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A53,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="I53" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A53,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>1</v>
+      </c>
+      <c r="J53" s="18" t="n">
+        <f aca="false">SUM(C53:I53)</f>
+        <v>5</v>
+      </c>
+      <c r="K53" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A53)</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="B54" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C54" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A54,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D54" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A54,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="E54" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A54,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F54" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A54,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G54" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A54,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H54" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A54,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I54" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A54,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J54" s="18" t="n">
+        <f aca="false">SUM(C54:I54)</f>
+        <v>3</v>
+      </c>
+      <c r="K54" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A54)</f>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B55" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C55" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A55,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D55" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A55,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E55" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A55,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F55" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A55,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G55" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A55,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>2</v>
+      </c>
+      <c r="H55" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A55,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I55" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A55,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J55" s="18" t="n">
+        <f aca="false">SUM(C55:I55)</f>
+        <v>2</v>
+      </c>
+      <c r="K55" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A55)</f>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C56" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A56,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D56" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A56,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E56" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A56,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F56" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A56,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G56" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A56,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H56" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A56,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I56" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A56,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J56" s="18" t="n">
+        <f aca="false">SUM(C56:I56)</f>
+        <v>2</v>
+      </c>
+      <c r="K56" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A56)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C57" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A57,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D57" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A57,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="E57" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A57,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F57" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A57,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G57" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A57,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H57" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A57,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I57" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A57,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J57" s="18" t="n">
+        <f aca="false">SUM(C57:I57)</f>
+        <v>3</v>
+      </c>
+      <c r="K57" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A57)</f>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="B58" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C58" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A58,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D58" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A58,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="E58" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A58,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F58" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A58,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G58" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A58,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H58" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A58,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I58" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A58,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J58" s="18" t="n">
+        <f aca="false">SUM(C58:I58)</f>
+        <v>3</v>
+      </c>
+      <c r="K58" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A58)</f>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="B59" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C59" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A59,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>0</v>
+      </c>
+      <c r="D59" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A59,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="E59" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A59,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="F59" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A59,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="G59" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A59,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="H59" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A59,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I59" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A59,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J59" s="18" t="n">
+        <f aca="false">SUM(C59:I59)</f>
+        <v>2</v>
+      </c>
+      <c r="K59" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A59)</f>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C60" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A60,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"5 x 10 cm (frente e verso)")</f>
+        <v>1</v>
+      </c>
+      <c r="D60" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A60,'Por Fragrância'!$D$5:$D$192,"Transparente",'Por Fragrância'!$E$5:$E$192,"6,5 x 5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="E60" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A60,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"13 x 5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="F60" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A60,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"18 x 6,5 cm")</f>
+        <v>1</v>
+      </c>
+      <c r="G60" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A60,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"22 x 8 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="H60" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A60,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"28 x 10,5 cm")</f>
+        <v>0</v>
+      </c>
+      <c r="I60" s="17" t="n">
+        <f aca="false">COUNTIFS('Por Fragrância'!$A$5:$A$192,$A60,'Por Fragrância'!$D$5:$D$192,"Vinil ou Bopp",'Por Fragrância'!$E$5:$E$192,"A definir")</f>
+        <v>0</v>
+      </c>
+      <c r="J60" s="18" t="n">
+        <f aca="false">SUM(C60:I60)</f>
+        <v>3</v>
+      </c>
+      <c r="K60" s="18" t="n">
+        <f aca="false">SUMIFS('Por Fragrância'!$J$5:$J$192,'Por Fragrância'!$A$5:$A$192,$A60)</f>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="B61" s="12"/>
+      <c r="C61" s="18" t="n">
+        <f aca="false">SUBTOTAL(9,C5:C60)</f>
+        <v>17</v>
+      </c>
+      <c r="D61" s="18" t="n">
+        <f aca="false">SUBTOTAL(9,D5:D60)</f>
+        <v>24</v>
+      </c>
+      <c r="E61" s="18" t="n">
+        <f aca="false">SUBTOTAL(9,E5:E60)</f>
+        <v>31</v>
+      </c>
+      <c r="F61" s="18" t="n">
+        <f aca="false">SUBTOTAL(9,F5:F60)</f>
+        <v>28</v>
+      </c>
+      <c r="G61" s="18" t="n">
+        <f aca="false">SUBTOTAL(9,G5:G60)</f>
+        <v>60</v>
+      </c>
+      <c r="H61" s="18" t="n">
+        <f aca="false">SUBTOTAL(9,H5:H60)</f>
+        <v>18</v>
+      </c>
+      <c r="I61" s="18" t="n">
+        <f aca="false">SUBTOTAL(9,I5:I60)</f>
+        <v>10</v>
+      </c>
+      <c r="J61" s="18" t="n">
+        <f aca="false">SUBTOTAL(9,J5:J60)</f>
+        <v>188</v>
+      </c>
+      <c r="K61" s="18" t="n">
+        <f aca="false">SUBTOTAL(9,K5:K60)</f>
+        <v>8332</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:K60"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:J195"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -7827,12 +10457,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7852,19 +10482,19 @@
         <v>10</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>98</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7919,7 +10549,7 @@
         <v>21</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>15</v>
@@ -8339,7 +10969,7 @@
         <v>21</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>15</v>
@@ -8673,36 +11303,36 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17" t="s">
+      <c r="A28" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="B28" s="17" t="s">
+      <c r="B28" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C28" s="17" t="n">
+      <c r="C28" s="19" t="n">
         <v>250</v>
       </c>
-      <c r="D28" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="E28" s="17" t="s">
+      <c r="D28" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="E28" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="F28" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="G28" s="17" t="s">
+      <c r="F28" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="G28" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="H28" s="18" t="n">
+      <c r="H28" s="20" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$A$5:$A$212,$A28,Rótulos!$B$5:$B$212,$B28,Rótulos!$C$5:$C$212,$C28,Rótulos!$H$5:$H$212,$D28,Rótulos!$I$5:$I$212,$E28,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>2</v>
       </c>
-      <c r="I28" s="18" t="n">
+      <c r="I28" s="20" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$A$5:$A$212,$A28,Rótulos!$B$5:$B$212,$B28,Rótulos!$C$5:$C$212,$C28,Rótulos!$H$5:$H$212,$D28,Rótulos!$I$5:$I$212,$E28,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>36</v>
       </c>
-      <c r="J28" s="19" t="n">
+      <c r="J28" s="21" t="n">
         <f aca="false">H28+I28</f>
         <v>38</v>
       </c>
@@ -8864,7 +11494,7 @@
         <v>21</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G33" s="4" t="s">
         <v>15</v>
@@ -8988,36 +11618,36 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="17" t="s">
+      <c r="A37" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="B37" s="17" t="s">
+      <c r="B37" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C37" s="17" t="n">
+      <c r="C37" s="19" t="n">
         <v>500</v>
       </c>
-      <c r="D37" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="E37" s="17" t="s">
+      <c r="D37" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="E37" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="F37" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="G37" s="17" t="s">
+      <c r="F37" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="G37" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="H37" s="18" t="n">
+      <c r="H37" s="20" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$A$5:$A$212,$A37,Rótulos!$B$5:$B$212,$B37,Rótulos!$C$5:$C$212,$C37,Rótulos!$H$5:$H$212,$D37,Rótulos!$I$5:$I$212,$E37,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>10</v>
       </c>
-      <c r="I37" s="18" t="n">
+      <c r="I37" s="20" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$A$5:$A$212,$A37,Rótulos!$B$5:$B$212,$B37,Rótulos!$C$5:$C$212,$C37,Rótulos!$H$5:$H$212,$D37,Rótulos!$I$5:$I$212,$E37,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>40</v>
       </c>
-      <c r="J37" s="19" t="n">
+      <c r="J37" s="21" t="n">
         <f aca="false">H37+I37</f>
         <v>50</v>
       </c>
@@ -9214,7 +11844,7 @@
         <v>21</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G43" s="4" t="s">
         <v>15</v>
@@ -9529,7 +12159,7 @@
         <v>21</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G52" s="4" t="s">
         <v>15</v>
@@ -9949,7 +12579,7 @@
         <v>21</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G64" s="4" t="s">
         <v>15</v>
@@ -10143,36 +12773,36 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="17" t="s">
+      <c r="A70" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="B70" s="17" t="s">
+      <c r="B70" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C70" s="17" t="n">
+      <c r="C70" s="19" t="n">
         <v>250</v>
       </c>
-      <c r="D70" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="E70" s="17" t="s">
+      <c r="D70" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="E70" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="F70" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="G70" s="17" t="s">
+      <c r="F70" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="G70" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="H70" s="18" t="n">
+      <c r="H70" s="20" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$A$5:$A$212,$A70,Rótulos!$B$5:$B$212,$B70,Rótulos!$C$5:$C$212,$C70,Rótulos!$H$5:$H$212,$D70,Rótulos!$I$5:$I$212,$E70,Rótulos!$F$5:$F$212,"B2C")</f>
         <v>2</v>
       </c>
-      <c r="I70" s="18" t="n">
+      <c r="I70" s="20" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$A$5:$A$212,$A70,Rótulos!$B$5:$B$212,$B70,Rótulos!$C$5:$C$212,$C70,Rótulos!$H$5:$H$212,$D70,Rótulos!$I$5:$I$212,$E70,Rótulos!$F$5:$F$212,"B2B")</f>
         <v>80</v>
       </c>
-      <c r="J70" s="19" t="n">
+      <c r="J70" s="21" t="n">
         <f aca="false">H70+I70</f>
         <v>82</v>
       </c>
@@ -10334,7 +12964,7 @@
         <v>21</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G75" s="4" t="s">
         <v>15</v>
@@ -10544,7 +13174,7 @@
         <v>21</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G81" s="4" t="s">
         <v>15</v>
@@ -12189,7 +14819,7 @@
         <v>21</v>
       </c>
       <c r="F128" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G128" s="4" t="s">
         <v>15</v>
@@ -12294,7 +14924,7 @@
         <v>21</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G131" s="4" t="s">
         <v>15</v>
@@ -12714,7 +15344,7 @@
         <v>21</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G143" s="4" t="s">
         <v>15</v>
@@ -13099,7 +15729,7 @@
         <v>21</v>
       </c>
       <c r="F154" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G154" s="4" t="s">
         <v>15</v>
@@ -13344,7 +15974,7 @@
         <v>21</v>
       </c>
       <c r="F161" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G161" s="4" t="s">
         <v>15</v>
@@ -13869,7 +16499,7 @@
         <v>21</v>
       </c>
       <c r="F176" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G176" s="4" t="s">
         <v>15</v>
@@ -14114,7 +16744,7 @@
         <v>21</v>
       </c>
       <c r="F183" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G183" s="4" t="s">
         <v>15</v>
@@ -14219,7 +16849,7 @@
         <v>21</v>
       </c>
       <c r="F186" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G186" s="4" t="s">
         <v>15</v>
@@ -14394,7 +17024,7 @@
         <v>21</v>
       </c>
       <c r="F191" s="4" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="G191" s="4" t="s">
         <v>15</v>
@@ -14466,7 +17096,7 @@
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="2" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -14483,7 +17113,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -14498,17 +17128,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>4</v>
@@ -14517,7 +17147,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>15</v>
@@ -14540,7 +17170,7 @@
         <v>17</v>
       </c>
       <c r="D5" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A5,Rótulos!$C$5:$C$212,$B5,Rótulos!$I$5:$I$212,$C5)</f>
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A5,'Por Fragrância'!$C$5:$C$192,$B5,'Por Fragrância'!$E$5:$E$192,$C5)</f>
         <v>24</v>
       </c>
       <c r="E5" s="15" t="n">
@@ -14567,8 +17197,8 @@
         <v>21</v>
       </c>
       <c r="D6" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A6,Rótulos!$C$5:$C$212,$B6,Rótulos!$I$5:$I$212,$C6)</f>
-        <v>34</v>
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A6,'Por Fragrância'!$C$5:$C$192,$B6,'Por Fragrância'!$E$5:$E$192,$C6)</f>
+        <v>17</v>
       </c>
       <c r="E6" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A6,Rótulos!$C$5:$C$212,$B6,Rótulos!$I$5:$I$212,$C6,Rótulos!$F$5:$F$212,"B2C")</f>
@@ -14594,7 +17224,7 @@
         <v>34</v>
       </c>
       <c r="D7" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A7,Rótulos!$C$5:$C$212,$B7,Rótulos!$I$5:$I$212,$C7)</f>
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A7,'Por Fragrância'!$C$5:$C$192,$B7,'Por Fragrância'!$E$5:$E$192,$C7)</f>
         <v>31</v>
       </c>
       <c r="E7" s="15" t="n">
@@ -14621,7 +17251,7 @@
         <v>25</v>
       </c>
       <c r="D8" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A8,Rótulos!$C$5:$C$212,$B8,Rótulos!$I$5:$I$212,$C8)</f>
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A8,'Por Fragrância'!$C$5:$C$192,$B8,'Por Fragrância'!$E$5:$E$192,$C8)</f>
         <v>6</v>
       </c>
       <c r="E8" s="15" t="n">
@@ -14648,7 +17278,7 @@
         <v>106</v>
       </c>
       <c r="D9" s="15" t="n">
-        <f aca="false">SUMPRODUCT((Rótulos!$I$5:$I$212="")*(Rótulos!$H$5:$H$212=$A9)*(Rótulos!$C$5:$C$212=$B9))</f>
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A9,'Por Fragrância'!$C$5:$C$192,$B9,'Por Fragrância'!$E$5:$E$192,$C9)</f>
         <v>6</v>
       </c>
       <c r="E9" s="15" t="n">
@@ -14675,7 +17305,7 @@
         <v>106</v>
       </c>
       <c r="D10" s="15" t="n">
-        <f aca="false">SUMPRODUCT((Rótulos!$I$5:$I$212="")*(Rótulos!$H$5:$H$212=$A10)*(Rótulos!$C$5:$C$212=$B10))</f>
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A10,'Por Fragrância'!$C$5:$C$192,$B10,'Por Fragrância'!$E$5:$E$192,$C10)</f>
         <v>1</v>
       </c>
       <c r="E10" s="15" t="n">
@@ -14702,8 +17332,8 @@
         <v>25</v>
       </c>
       <c r="D11" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A11,Rótulos!$C$5:$C$212,$B11,Rótulos!$I$5:$I$212,$C11)</f>
-        <v>24</v>
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A11,'Por Fragrância'!$C$5:$C$192,$B11,'Por Fragrância'!$E$5:$E$192,$C11)</f>
+        <v>22</v>
       </c>
       <c r="E11" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A11,Rótulos!$C$5:$C$212,$B11,Rótulos!$I$5:$I$212,$C11,Rótulos!$F$5:$F$212,"B2C")</f>
@@ -14729,7 +17359,7 @@
         <v>31</v>
       </c>
       <c r="D12" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A12,Rótulos!$C$5:$C$212,$B12,Rótulos!$I$5:$I$212,$C12)</f>
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A12,'Por Fragrância'!$C$5:$C$192,$B12,'Por Fragrância'!$E$5:$E$192,$C12)</f>
         <v>26</v>
       </c>
       <c r="E12" s="15" t="n">
@@ -14756,8 +17386,8 @@
         <v>31</v>
       </c>
       <c r="D13" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A13,Rótulos!$C$5:$C$212,$B13,Rótulos!$I$5:$I$212,$C13)</f>
-        <v>35</v>
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A13,'Por Fragrância'!$C$5:$C$192,$B13,'Por Fragrância'!$E$5:$E$192,$C13)</f>
+        <v>34</v>
       </c>
       <c r="E13" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$H$5:$H$212,$A13,Rótulos!$C$5:$C$212,$B13,Rótulos!$I$5:$I$212,$C13,Rótulos!$F$5:$F$212,"B2C")</f>
@@ -14783,7 +17413,7 @@
         <v>32</v>
       </c>
       <c r="D14" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$H$5:$H$212,$A14,Rótulos!$C$5:$C$212,$B14,Rótulos!$I$5:$I$212,$C14)</f>
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A14,'Por Fragrância'!$C$5:$C$192,$B14,'Por Fragrância'!$E$5:$E$192,$C14)</f>
         <v>18</v>
       </c>
       <c r="E14" s="15" t="n">
@@ -14810,7 +17440,7 @@
         <v>106</v>
       </c>
       <c r="D15" s="15" t="n">
-        <f aca="false">SUMPRODUCT((Rótulos!$I$5:$I$212="")*(Rótulos!$H$5:$H$212=$A15)*(Rótulos!$C$5:$C$212=$B15))</f>
+        <f aca="false">COUNTIFS('Por Fragrância'!$D$5:$D$192,$A15,'Por Fragrância'!$C$5:$C$192,$B15,'Por Fragrância'!$E$5:$E$192,$C15)</f>
         <v>3</v>
       </c>
       <c r="E15" s="15" t="n">
@@ -14834,7 +17464,7 @@
       <c r="C16" s="16"/>
       <c r="D16" s="16" t="n">
         <f aca="false">SUM(D5:D15)</f>
-        <v>208</v>
+        <v>188</v>
       </c>
       <c r="E16" s="16" t="n">
         <f aca="false">SUM(E5:E15)</f>
@@ -14851,18 +17481,18 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>15</v>
@@ -14882,7 +17512,7 @@
         <v>24</v>
       </c>
       <c r="C20" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$I$5:$I$212,$A20,Rótulos!$H$5:$H$212,$B20)</f>
+        <f aca="false">COUNTIFS('Por Fragrância'!$E$5:$E$192,$A20,'Por Fragrância'!$D$5:$D$192,$B20)</f>
         <v>31</v>
       </c>
       <c r="D20" s="15" t="n">
@@ -14906,8 +17536,8 @@
         <v>24</v>
       </c>
       <c r="C21" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$I$5:$I$212,$A21,Rótulos!$H$5:$H$212,$B21)</f>
-        <v>30</v>
+        <f aca="false">COUNTIFS('Por Fragrância'!$E$5:$E$192,$A21,'Por Fragrância'!$D$5:$D$192,$B21)</f>
+        <v>28</v>
       </c>
       <c r="D21" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A21,Rótulos!$H$5:$H$212,$B21,Rótulos!$F$5:$F$212,"B2C")</f>
@@ -14930,8 +17560,8 @@
         <v>24</v>
       </c>
       <c r="C22" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$I$5:$I$212,$A22,Rótulos!$H$5:$H$212,$B22)</f>
-        <v>61</v>
+        <f aca="false">COUNTIFS('Por Fragrância'!$E$5:$E$192,$A22,'Por Fragrância'!$D$5:$D$192,$B22)</f>
+        <v>60</v>
       </c>
       <c r="D22" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A22,Rótulos!$H$5:$H$212,$B22,Rótulos!$F$5:$F$212,"B2C")</f>
@@ -14954,7 +17584,7 @@
         <v>24</v>
       </c>
       <c r="C23" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$I$5:$I$212,$A23,Rótulos!$H$5:$H$212,$B23)</f>
+        <f aca="false">COUNTIFS('Por Fragrância'!$E$5:$E$192,$A23,'Por Fragrância'!$D$5:$D$192,$B23)</f>
         <v>18</v>
       </c>
       <c r="D23" s="15" t="n">
@@ -14978,8 +17608,8 @@
         <v>16</v>
       </c>
       <c r="C24" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$I$5:$I$212,$A24,Rótulos!$H$5:$H$212,$B24)</f>
-        <v>34</v>
+        <f aca="false">COUNTIFS('Por Fragrância'!$E$5:$E$192,$A24,'Por Fragrância'!$D$5:$D$192,$B24)</f>
+        <v>17</v>
       </c>
       <c r="D24" s="15" t="n">
         <f aca="false">SUMIFS(Rótulos!$G$5:$G$212,Rótulos!$I$5:$I$212,$A24,Rótulos!$H$5:$H$212,$B24,Rótulos!$F$5:$F$212,"B2C")</f>
@@ -15002,7 +17632,7 @@
         <v>16</v>
       </c>
       <c r="C25" s="15" t="n">
-        <f aca="false">COUNTIFS(Rótulos!$I$5:$I$212,$A25,Rótulos!$H$5:$H$212,$B25)</f>
+        <f aca="false">COUNTIFS('Por Fragrância'!$E$5:$E$192,$A25,'Por Fragrância'!$D$5:$D$192,$B25)</f>
         <v>24</v>
       </c>
       <c r="D25" s="15" t="n">
@@ -15026,7 +17656,7 @@
         <v>24</v>
       </c>
       <c r="C26" s="15" t="n">
-        <f aca="false">SUMPRODUCT((Rótulos!$I$5:$I$212="")*(Rótulos!$H$5:$H$212=$B26))</f>
+        <f aca="false">COUNTIFS('Por Fragrância'!$E$5:$E$192,$A26,'Por Fragrância'!$D$5:$D$192,$B26)</f>
         <v>10</v>
       </c>
       <c r="D26" s="15" t="n">
@@ -15049,7 +17679,7 @@
       <c r="B27" s="16"/>
       <c r="C27" s="16" t="n">
         <f aca="false">SUM(C20:C26)</f>
-        <v>208</v>
+        <v>188</v>
       </c>
       <c r="D27" s="16" t="n">
         <f aca="false">SUM(D20:D26)</f>
@@ -15075,7 +17705,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -15092,12 +17722,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15111,13 +17741,13 @@
         <v>4</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15479,7 +18109,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>33</v>
@@ -16109,7 +18739,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>29</v>
@@ -16277,10 +18907,10 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="C60" s="4" t="n">
         <v>500</v>

</xml_diff>